<commit_message>
xlsx: ISRUC rotation and the TUEV spatial-head safety check
ISRUC rotation kappa 0.7104 against product 0.6952 (+0.015) and raw 0.7013
(+0.009). Rotation is now >= product on five of the six corpora it has run on.

TUEV spatial head 0.6520 against the mean head 0.7076 -- it COSTS 0.056. This
was the tier-1 safety check and it fails, which is what the mechanism predicted:
tier-1 labels (seizure, artifact, sleep stage) are spatially diffuse or are
properties of the whole recording, so keeping electrode identity buys nothing
and spends parameters. head: spatial must stay corpus-conditional, like
patch_len already is -- it is not a global default.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/PACLock_baseline_matrix_filled.xlsx
+++ b/results/PACLock_baseline_matrix_filled.xlsx
@@ -11275,7 +11275,11 @@
           <t>0.6449±0.0000 (1)</t>
         </is>
       </c>
-      <c r="H11" s="313" t="n"/>
+      <c r="H11" s="315" t="inlineStr">
+        <is>
+          <t>0.7104±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="I11" s="315" t="inlineStr">
         <is>
           <t>0.2961±0.0000 (1)</t>
@@ -11331,7 +11335,11 @@
         </is>
       </c>
       <c r="C13" s="313" t="n"/>
-      <c r="D13" s="313" t="n"/>
+      <c r="D13" s="315" t="inlineStr">
+        <is>
+          <t>0.6520±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="E13" s="313" t="n"/>
       <c r="F13" s="313" t="n"/>
       <c r="G13" s="313" t="n"/>

</xml_diff>

<commit_message>
xlsx: PACLock (hybrid) row in every main sheet
Requested by Zhizhe: the plain hybrid joins the nine per-corpus main sheets as
a fourth PACLock row under pt-large, no longer only in the ablation sheet.

Same column conventions as the sheet: metric cells from result.json, the three
delta columns recomputed against the scratch / pt-base / pt-large rows AS
DISPLAYED (read back from the sheet so the arithmetic cannot diverge from it).
A single-seed cell is written as "value (1 seed)" in italics -- the count is
never dropped -- and corpora without a hybrid run carry an em-dash placeholder
so "not run" stays distinguishable from "ran and failed".

What the row shows where it exists (all 1 seed): CHB-MIT 0.7473, +0.2009 over
scratch and +0.0643 over the previous best (pt-base) -- the project best.
TUEV 0.6951. TUSZ 0.6299. BCI-IV-2a 0.3912.

The ablation sheet gains the hybrid family rows (plain / +gate / +attn) too.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/PACLock_baseline_matrix_filled.xlsx
+++ b/results/PACLock_baseline_matrix_filled.xlsx
@@ -28,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="44">
+  <fonts count="45">
     <font>
       <name val="Calibri"/>
       <color indexed="8"/>
@@ -259,6 +259,10 @@
     <font>
       <i val="1"/>
       <color rgb="00808080"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="22">
@@ -1234,7 +1238,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="318">
+  <cellXfs count="322">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -2141,6 +2145,18 @@
     </xf>
     <xf numFmtId="0" fontId="34" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="68" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="10" borderId="68" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="10" borderId="68" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="68" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3519,7 +3535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="219" min="1" max="4"/>
@@ -4258,15 +4274,55 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1" s="220"/>
-    <row r="22" ht="22" customHeight="1" s="220">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21" ht="32" customHeight="1" s="220">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="318" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="319" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="D21" s="320" t="inlineStr">
+        <is>
+          <t>0.3912 (1 seed)</t>
+        </is>
+      </c>
+      <c r="E21" s="320" t="inlineStr">
+        <is>
+          <t>0.1883 (1 seed)</t>
+        </is>
+      </c>
+      <c r="F21" s="320" t="inlineStr">
+        <is>
+          <t>0.3796 (1 seed)</t>
+        </is>
+      </c>
+      <c r="G21" s="320" t="inlineStr">
+        <is>
+          <t>+0.0324</t>
+        </is>
+      </c>
+      <c r="H21" s="321" t="inlineStr">
+        <is>
+          <t>+0.0260</t>
+        </is>
+      </c>
+      <c r="I21" s="321" t="inlineStr">
+        <is>
+          <t>-0.0210</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" s="220"/>
+    <row r="23" ht="38" customHeight="1" s="220">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="38" customHeight="1" s="220"/>
     <row r="24" ht="38" customHeight="1" s="220"/>
     <row r="25" ht="38" customHeight="1" s="220"/>
     <row r="26" ht="38" customHeight="1" s="220"/>
@@ -10910,7 +10966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="220" min="1" max="1"/>
@@ -11255,52 +11311,32 @@
       </c>
       <c r="B11" s="312" t="inlineStr">
         <is>
-          <t>rotation(耦合只旋转不缩放)</t>
-        </is>
-      </c>
-      <c r="C11" s="315" t="inlineStr">
-        <is>
-          <t>0.8806±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="D11" s="313" t="inlineStr">
-        <is>
-          <t>0.7328±0.0161 (3)</t>
+          <t>hybrid(raw 行 + 交互行并列)</t>
+        </is>
+      </c>
+      <c r="C11" s="313" t="n"/>
+      <c r="D11" s="315" t="inlineStr">
+        <is>
+          <t>0.6951±0.0000 (1)</t>
         </is>
       </c>
       <c r="E11" s="315" t="inlineStr">
         <is>
-          <t>0.6884±0.0000 (1)</t>
+          <t>0.6299±0.0000 (1)</t>
         </is>
       </c>
       <c r="F11" s="315" t="inlineStr">
         <is>
-          <t>0.5100±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="G11" s="315" t="inlineStr">
-        <is>
-          <t>0.6449±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="H11" s="315" t="inlineStr">
-        <is>
-          <t>0.7104±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="I11" s="315" t="inlineStr">
-        <is>
-          <t>0.2961±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="J11" s="315" t="inlineStr">
-        <is>
-          <t>0.1514±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="K11" s="313" t="inlineStr">
-        <is>
-          <t>0.3708±0.0092 (3)</t>
+          <t>0.7473±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="G11" s="313" t="n"/>
+      <c r="H11" s="313" t="n"/>
+      <c r="I11" s="313" t="n"/>
+      <c r="J11" s="313" t="n"/>
+      <c r="K11" s="315" t="inlineStr">
+        <is>
+          <t>0.3912±0.0000 (1)</t>
         </is>
       </c>
       <c r="L11" s="313" t="n"/>
@@ -11309,62 +11345,62 @@
       <c r="A12" s="312" t="inlineStr"/>
       <c r="B12" s="312" t="inlineStr">
         <is>
-          <t>rotation(跑在 PAC 协议数据上,与上行不可比)</t>
+          <t>hybrid + 逐频带可学门</t>
         </is>
       </c>
       <c r="C12" s="313" t="n"/>
-      <c r="D12" s="313" t="n"/>
-      <c r="E12" s="313" t="n"/>
+      <c r="D12" s="315" t="inlineStr">
+        <is>
+          <t>0.6929±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="E12" s="315" t="inlineStr">
+        <is>
+          <t>0.6455±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="F12" s="313" t="n"/>
       <c r="G12" s="313" t="n"/>
       <c r="H12" s="313" t="n"/>
       <c r="I12" s="313" t="n"/>
-      <c r="J12" s="315" t="inlineStr">
-        <is>
-          <t>0.1098±0.0000 (1)</t>
-        </is>
-      </c>
+      <c r="J12" s="313" t="n"/>
       <c r="K12" s="315" t="inlineStr">
         <is>
-          <t>0.2724±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="L12" s="315" t="inlineStr">
-        <is>
-          <t>0.5568±0.0000 (1)</t>
-        </is>
-      </c>
+          <t>0.3970±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="L12" s="313" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="312" t="inlineStr"/>
       <c r="B13" s="312" t="inlineStr">
         <is>
-          <t>spatial 头(保留电极身份)</t>
+          <t>hybrid + attn 头</t>
         </is>
       </c>
       <c r="C13" s="313" t="n"/>
       <c r="D13" s="315" t="inlineStr">
         <is>
-          <t>0.6520±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="E13" s="313" t="n"/>
-      <c r="F13" s="313" t="n"/>
+          <t>0.6814±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="E13" s="315" t="inlineStr">
+        <is>
+          <t>0.6306±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="F13" s="315" t="inlineStr">
+        <is>
+          <t>0.7200±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="G13" s="313" t="n"/>
       <c r="H13" s="313" t="n"/>
-      <c r="I13" s="315" t="inlineStr">
-        <is>
-          <t>0.3560±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="J13" s="315" t="inlineStr">
-        <is>
-          <t>0.1514±0.0000 (1)</t>
-        </is>
-      </c>
+      <c r="I13" s="313" t="n"/>
+      <c r="J13" s="313" t="n"/>
       <c r="K13" s="315" t="inlineStr">
         <is>
-          <t>0.4144±0.0000 (1)</t>
+          <t>0.3542±0.0000 (1)</t>
         </is>
       </c>
       <c r="L13" s="313" t="n"/>
@@ -11373,136 +11409,116 @@
       <c r="A14" s="312" t="inlineStr"/>
       <c r="B14" s="312" t="inlineStr">
         <is>
-          <t>rotation + spatial 头</t>
-        </is>
-      </c>
-      <c r="C14" s="313" t="n"/>
-      <c r="D14" s="313" t="n"/>
-      <c r="E14" s="313" t="n"/>
-      <c r="F14" s="313" t="n"/>
-      <c r="G14" s="313" t="n"/>
-      <c r="H14" s="313" t="n"/>
+          <t>rotation(耦合只旋转不缩放)</t>
+        </is>
+      </c>
+      <c r="C14" s="315" t="inlineStr">
+        <is>
+          <t>0.8806±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="D14" s="313" t="inlineStr">
+        <is>
+          <t>0.7328±0.0161 (3)</t>
+        </is>
+      </c>
+      <c r="E14" s="315" t="inlineStr">
+        <is>
+          <t>0.6884±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="F14" s="315" t="inlineStr">
+        <is>
+          <t>0.5100±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="G14" s="315" t="inlineStr">
+        <is>
+          <t>0.6449±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="H14" s="315" t="inlineStr">
+        <is>
+          <t>0.7104±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="I14" s="315" t="inlineStr">
         <is>
-          <t>0.3299±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="J14" s="313" t="n"/>
-      <c r="K14" s="315" t="inlineStr">
-        <is>
-          <t>0.4344±0.0000 (1)</t>
+          <t>0.2916±0.0063 (2)</t>
+        </is>
+      </c>
+      <c r="J14" s="315" t="inlineStr">
+        <is>
+          <t>0.1514±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="K14" s="313" t="inlineStr">
+        <is>
+          <t>0.3708±0.0092 (3)</t>
         </is>
       </c>
       <c r="L14" s="313" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="311" t="inlineStr">
-        <is>
-          <t>预训练</t>
-        </is>
-      </c>
+      <c r="A15" s="312" t="inlineStr"/>
       <c r="B15" s="312" t="inlineStr">
         <is>
-          <t>预训练 base(60k)</t>
-        </is>
-      </c>
-      <c r="C15" s="313" t="inlineStr">
-        <is>
-          <t>0.8841±0.0043 (3)</t>
-        </is>
-      </c>
-      <c r="D15" s="313" t="inlineStr">
-        <is>
-          <t>0.6730±0.0116 (3)</t>
-        </is>
-      </c>
-      <c r="E15" s="313" t="inlineStr">
-        <is>
-          <t>0.6398±0.0615 (3)</t>
-        </is>
-      </c>
-      <c r="F15" s="313" t="inlineStr">
-        <is>
-          <t>0.6830±0.0228 (3)</t>
-        </is>
-      </c>
-      <c r="G15" s="313" t="inlineStr">
-        <is>
-          <t>0.6651±0.0109 (3)</t>
-        </is>
-      </c>
-      <c r="H15" s="313" t="inlineStr">
-        <is>
-          <t>0.6934±0.0032 (3)</t>
-        </is>
-      </c>
-      <c r="I15" s="313" t="inlineStr">
-        <is>
-          <t>0.3059±0.0262 (3)</t>
-        </is>
-      </c>
-      <c r="J15" s="313" t="inlineStr">
-        <is>
-          <t>0.1540±0.0202 (3)</t>
-        </is>
-      </c>
-      <c r="K15" s="313" t="inlineStr">
-        <is>
-          <t>0.3652±0.0083 (3)</t>
-        </is>
-      </c>
-      <c r="L15" s="313" t="n"/>
+          <t>rotation(跑在 PAC 协议数据上,与上行不可比)</t>
+        </is>
+      </c>
+      <c r="C15" s="313" t="n"/>
+      <c r="D15" s="313" t="n"/>
+      <c r="E15" s="313" t="n"/>
+      <c r="F15" s="313" t="n"/>
+      <c r="G15" s="313" t="n"/>
+      <c r="H15" s="313" t="n"/>
+      <c r="I15" s="313" t="n"/>
+      <c r="J15" s="315" t="inlineStr">
+        <is>
+          <t>0.1098±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="K15" s="315" t="inlineStr">
+        <is>
+          <t>0.2724±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="L15" s="315" t="inlineStr">
+        <is>
+          <t>0.5568±0.0000 (1)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="312" t="inlineStr"/>
       <c r="B16" s="312" t="inlineStr">
         <is>
-          <t>预训练 large(60k)</t>
-        </is>
-      </c>
-      <c r="C16" s="313" t="inlineStr">
-        <is>
-          <t>0.8869±0.0069 (3)</t>
-        </is>
-      </c>
-      <c r="D16" s="313" t="inlineStr">
-        <is>
-          <t>0.6523±0.0302 (3)</t>
-        </is>
-      </c>
-      <c r="E16" s="313" t="inlineStr">
-        <is>
-          <t>0.6289±0.0297 (3)</t>
-        </is>
-      </c>
-      <c r="F16" s="313" t="inlineStr">
-        <is>
-          <t>0.6162±0.0467 (3)</t>
-        </is>
-      </c>
-      <c r="G16" s="313" t="inlineStr">
-        <is>
-          <t>0.6641±0.0044 (3)</t>
-        </is>
-      </c>
-      <c r="H16" s="313" t="inlineStr">
-        <is>
-          <t>0.6996±0.0153 (3)</t>
-        </is>
-      </c>
+          <t>spatial 头(保留电极身份)</t>
+        </is>
+      </c>
+      <c r="C16" s="313" t="n"/>
+      <c r="D16" s="315" t="inlineStr">
+        <is>
+          <t>0.6520±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="E16" s="313" t="n"/>
+      <c r="F16" s="313" t="n"/>
+      <c r="G16" s="313" t="n"/>
+      <c r="H16" s="313" t="n"/>
       <c r="I16" s="313" t="inlineStr">
         <is>
-          <t>0.3140±0.0094 (3)</t>
-        </is>
-      </c>
-      <c r="J16" s="313" t="inlineStr">
-        <is>
-          <t>0.1640±0.0155 (3)</t>
+          <t>0.3535±0.0047 (3)</t>
+        </is>
+      </c>
+      <c r="J16" s="315" t="inlineStr">
+        <is>
+          <t>0.1514±0.0000 (1)</t>
         </is>
       </c>
       <c r="K16" s="313" t="inlineStr">
         <is>
-          <t>0.4122±0.0166 (3)</t>
+          <t>0.4317±0.0153 (3)</t>
         </is>
       </c>
       <c r="L16" s="313" t="n"/>
@@ -11511,7 +11527,7 @@
       <c r="A17" s="312" t="inlineStr"/>
       <c r="B17" s="312" t="inlineStr">
         <is>
-          <t>raw tokenizer 预训练 large(60k)</t>
+          <t>rotation + spatial 头</t>
         </is>
       </c>
       <c r="C17" s="313" t="n"/>
@@ -11520,120 +11536,192 @@
       <c r="F17" s="313" t="n"/>
       <c r="G17" s="313" t="n"/>
       <c r="H17" s="313" t="n"/>
-      <c r="I17" s="313" t="inlineStr">
-        <is>
-          <t>0.3633±0.0349 (3)</t>
-        </is>
-      </c>
-      <c r="J17" s="315" t="inlineStr">
-        <is>
-          <t>0.1690±0.0018 (2)</t>
-        </is>
-      </c>
-      <c r="K17" s="313" t="inlineStr">
-        <is>
-          <t>0.4483±0.0031 (3)</t>
+      <c r="I17" s="315" t="inlineStr">
+        <is>
+          <t>0.3299±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J17" s="313" t="n"/>
+      <c r="K17" s="315" t="inlineStr">
+        <is>
+          <t>0.4344±0.0000 (1)</t>
         </is>
       </c>
       <c r="L17" s="313" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="312" t="inlineStr"/>
+      <c r="A18" s="311" t="inlineStr">
+        <is>
+          <t>预训练</t>
+        </is>
+      </c>
       <c r="B18" s="312" t="inlineStr">
         <is>
-          <t>预训练池剔除 TUSZ/CHB-MIT</t>
-        </is>
-      </c>
-      <c r="C18" s="313" t="n"/>
-      <c r="D18" s="313" t="n"/>
-      <c r="E18" s="315" t="inlineStr">
-        <is>
-          <t>0.6221±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="F18" s="315" t="inlineStr">
-        <is>
-          <t>0.6410±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="G18" s="313" t="n"/>
-      <c r="H18" s="313" t="n"/>
-      <c r="I18" s="313" t="n"/>
-      <c r="J18" s="313" t="n"/>
-      <c r="K18" s="313" t="n"/>
+          <t>预训练 base(60k)</t>
+        </is>
+      </c>
+      <c r="C18" s="313" t="inlineStr">
+        <is>
+          <t>0.8841±0.0043 (3)</t>
+        </is>
+      </c>
+      <c r="D18" s="313" t="inlineStr">
+        <is>
+          <t>0.6730±0.0116 (3)</t>
+        </is>
+      </c>
+      <c r="E18" s="313" t="inlineStr">
+        <is>
+          <t>0.6398±0.0615 (3)</t>
+        </is>
+      </c>
+      <c r="F18" s="313" t="inlineStr">
+        <is>
+          <t>0.6830±0.0228 (3)</t>
+        </is>
+      </c>
+      <c r="G18" s="313" t="inlineStr">
+        <is>
+          <t>0.6651±0.0109 (3)</t>
+        </is>
+      </c>
+      <c r="H18" s="313" t="inlineStr">
+        <is>
+          <t>0.6934±0.0032 (3)</t>
+        </is>
+      </c>
+      <c r="I18" s="313" t="inlineStr">
+        <is>
+          <t>0.3059±0.0262 (3)</t>
+        </is>
+      </c>
+      <c r="J18" s="313" t="inlineStr">
+        <is>
+          <t>0.1540±0.0202 (3)</t>
+        </is>
+      </c>
+      <c r="K18" s="313" t="inlineStr">
+        <is>
+          <t>0.3652±0.0083 (3)</t>
+        </is>
+      </c>
       <c r="L18" s="313" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="312" t="inlineStr"/>
       <c r="B19" s="312" t="inlineStr">
         <is>
-          <t>预训练 base,微调 patch_len=200</t>
-        </is>
-      </c>
-      <c r="C19" s="313" t="n"/>
+          <t>预训练 large(60k)</t>
+        </is>
+      </c>
+      <c r="C19" s="313" t="inlineStr">
+        <is>
+          <t>0.8869±0.0069 (3)</t>
+        </is>
+      </c>
       <c r="D19" s="313" t="inlineStr">
         <is>
-          <t>0.6793±0.0109 (3)</t>
-        </is>
-      </c>
-      <c r="E19" s="313" t="n"/>
-      <c r="F19" s="313" t="n"/>
-      <c r="G19" s="313" t="n"/>
-      <c r="H19" s="313" t="n"/>
-      <c r="I19" s="313" t="n"/>
-      <c r="J19" s="313" t="n"/>
-      <c r="K19" s="313" t="n"/>
+          <t>0.6523±0.0302 (3)</t>
+        </is>
+      </c>
+      <c r="E19" s="313" t="inlineStr">
+        <is>
+          <t>0.6289±0.0297 (3)</t>
+        </is>
+      </c>
+      <c r="F19" s="313" t="inlineStr">
+        <is>
+          <t>0.6162±0.0467 (3)</t>
+        </is>
+      </c>
+      <c r="G19" s="313" t="inlineStr">
+        <is>
+          <t>0.6641±0.0044 (3)</t>
+        </is>
+      </c>
+      <c r="H19" s="313" t="inlineStr">
+        <is>
+          <t>0.6996±0.0153 (3)</t>
+        </is>
+      </c>
+      <c r="I19" s="313" t="inlineStr">
+        <is>
+          <t>0.3140±0.0094 (3)</t>
+        </is>
+      </c>
+      <c r="J19" s="313" t="inlineStr">
+        <is>
+          <t>0.1640±0.0155 (3)</t>
+        </is>
+      </c>
+      <c r="K19" s="313" t="inlineStr">
+        <is>
+          <t>0.4122±0.0166 (3)</t>
+        </is>
+      </c>
       <c r="L19" s="313" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="312" t="inlineStr"/>
       <c r="B20" s="312" t="inlineStr">
         <is>
-          <t>早期微调配方(6k checkpoint)</t>
+          <t>raw tokenizer 预训练 large(60k)</t>
         </is>
       </c>
       <c r="C20" s="313" t="n"/>
       <c r="D20" s="313" t="n"/>
-      <c r="E20" s="313" t="n"/>
-      <c r="F20" s="313" t="n"/>
+      <c r="E20" s="315" t="inlineStr">
+        <is>
+          <t>0.5460±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="F20" s="315" t="inlineStr">
+        <is>
+          <t>0.6279±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="G20" s="313" t="n"/>
       <c r="H20" s="313" t="n"/>
-      <c r="I20" s="315" t="inlineStr">
-        <is>
-          <t>0.2690±0.0000 (1)</t>
+      <c r="I20" s="313" t="inlineStr">
+        <is>
+          <t>0.3633±0.0349 (3)</t>
         </is>
       </c>
       <c r="J20" s="315" t="inlineStr">
         <is>
-          <t>0.1279±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="K20" s="313" t="n"/>
+          <t>0.1690±0.0018 (2)</t>
+        </is>
+      </c>
+      <c r="K20" s="313" t="inlineStr">
+        <is>
+          <t>0.4483±0.0031 (3)</t>
+        </is>
+      </c>
       <c r="L20" s="313" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="312" t="inlineStr"/>
       <c r="B21" s="312" t="inlineStr">
         <is>
-          <t>早期微调配方 v2(6k checkpoint)</t>
+          <t>预训练池剔除 TUSZ/CHB-MIT</t>
         </is>
       </c>
       <c r="C21" s="313" t="n"/>
       <c r="D21" s="313" t="n"/>
-      <c r="E21" s="313" t="n"/>
-      <c r="F21" s="313" t="n"/>
+      <c r="E21" s="315" t="inlineStr">
+        <is>
+          <t>0.6221±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="F21" s="315" t="inlineStr">
+        <is>
+          <t>0.6410±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="G21" s="313" t="n"/>
       <c r="H21" s="313" t="n"/>
-      <c r="I21" s="315" t="inlineStr">
-        <is>
-          <t>0.2622±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="J21" s="315" t="inlineStr">
-        <is>
-          <t>0.1408±0.0000 (1)</t>
-        </is>
-      </c>
+      <c r="I21" s="313" t="n"/>
+      <c r="J21" s="313" t="n"/>
       <c r="K21" s="313" t="n"/>
       <c r="L21" s="313" t="n"/>
     </row>
@@ -11641,37 +11729,29 @@
       <c r="A22" s="312" t="inlineStr"/>
       <c r="B22" s="312" t="inlineStr">
         <is>
-          <t>早期微调配方 large(6k checkpoint)</t>
+          <t>预训练 base,微调 patch_len=200</t>
         </is>
       </c>
       <c r="C22" s="313" t="n"/>
-      <c r="D22" s="313" t="n"/>
+      <c r="D22" s="313" t="inlineStr">
+        <is>
+          <t>0.6793±0.0109 (3)</t>
+        </is>
+      </c>
       <c r="E22" s="313" t="n"/>
       <c r="F22" s="313" t="n"/>
       <c r="G22" s="313" t="n"/>
       <c r="H22" s="313" t="n"/>
-      <c r="I22" s="315" t="inlineStr">
-        <is>
-          <t>0.2716±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="J22" s="315" t="inlineStr">
-        <is>
-          <t>0.1381±0.0000 (1)</t>
-        </is>
-      </c>
+      <c r="I22" s="313" t="n"/>
+      <c r="J22" s="313" t="n"/>
       <c r="K22" s="313" t="n"/>
       <c r="L22" s="313" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="311" t="inlineStr">
-        <is>
-          <t>容量阶梯</t>
-        </is>
-      </c>
+      <c r="A23" s="312" t="inlineStr"/>
       <c r="B23" s="312" t="inlineStr">
         <is>
-          <t>raw,d_model 32</t>
+          <t>早期微调配方(6k checkpoint)</t>
         </is>
       </c>
       <c r="C23" s="313" t="n"/>
@@ -11680,24 +11760,24 @@
       <c r="F23" s="313" t="n"/>
       <c r="G23" s="313" t="n"/>
       <c r="H23" s="313" t="n"/>
-      <c r="I23" s="313" t="inlineStr">
-        <is>
-          <t>0.2613±0.0100 (3)</t>
-        </is>
-      </c>
-      <c r="J23" s="313" t="n"/>
-      <c r="K23" s="313" t="inlineStr">
-        <is>
-          <t>0.2617±0.0019 (3)</t>
-        </is>
-      </c>
+      <c r="I23" s="315" t="inlineStr">
+        <is>
+          <t>0.2690±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J23" s="315" t="inlineStr">
+        <is>
+          <t>0.1279±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="K23" s="313" t="n"/>
       <c r="L23" s="313" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="312" t="inlineStr"/>
       <c r="B24" s="312" t="inlineStr">
         <is>
-          <t>raw,d_model 64</t>
+          <t>早期微调配方 v2(6k checkpoint)</t>
         </is>
       </c>
       <c r="C24" s="313" t="n"/>
@@ -11706,24 +11786,24 @@
       <c r="F24" s="313" t="n"/>
       <c r="G24" s="313" t="n"/>
       <c r="H24" s="313" t="n"/>
-      <c r="I24" s="313" t="inlineStr">
-        <is>
-          <t>0.3129±0.0121 (3)</t>
-        </is>
-      </c>
-      <c r="J24" s="313" t="n"/>
-      <c r="K24" s="313" t="inlineStr">
-        <is>
-          <t>0.2780±0.0100 (3)</t>
-        </is>
-      </c>
+      <c r="I24" s="315" t="inlineStr">
+        <is>
+          <t>0.2622±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J24" s="315" t="inlineStr">
+        <is>
+          <t>0.1408±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="K24" s="313" t="n"/>
       <c r="L24" s="313" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="312" t="inlineStr"/>
       <c r="B25" s="312" t="inlineStr">
         <is>
-          <t>raw,d_model 256</t>
+          <t>早期微调配方 large(6k checkpoint)</t>
         </is>
       </c>
       <c r="C25" s="313" t="n"/>
@@ -11732,24 +11812,28 @@
       <c r="F25" s="313" t="n"/>
       <c r="G25" s="313" t="n"/>
       <c r="H25" s="313" t="n"/>
-      <c r="I25" s="313" t="inlineStr">
-        <is>
-          <t>0.4159±0.0529 (3)</t>
-        </is>
-      </c>
-      <c r="J25" s="313" t="n"/>
-      <c r="K25" s="313" t="inlineStr">
-        <is>
-          <t>0.4437±0.0192 (3)</t>
-        </is>
-      </c>
+      <c r="I25" s="315" t="inlineStr">
+        <is>
+          <t>0.2716±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J25" s="315" t="inlineStr">
+        <is>
+          <t>0.1381±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="K25" s="313" t="n"/>
       <c r="L25" s="313" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="312" t="inlineStr"/>
+      <c r="A26" s="311" t="inlineStr">
+        <is>
+          <t>容量阶梯</t>
+        </is>
+      </c>
       <c r="B26" s="312" t="inlineStr">
         <is>
-          <t>raw,加宽</t>
+          <t>raw,d_model 32</t>
         </is>
       </c>
       <c r="C26" s="313" t="n"/>
@@ -11760,13 +11844,13 @@
       <c r="H26" s="313" t="n"/>
       <c r="I26" s="313" t="inlineStr">
         <is>
-          <t>0.4093±0.0425 (3)</t>
+          <t>0.2613±0.0100 (3)</t>
         </is>
       </c>
       <c r="J26" s="313" t="n"/>
-      <c r="K26" s="315" t="inlineStr">
-        <is>
-          <t>0.4261±0.0085 (2)</t>
+      <c r="K26" s="313" t="inlineStr">
+        <is>
+          <t>0.2617±0.0019 (3)</t>
         </is>
       </c>
       <c r="L26" s="313" t="n"/>
@@ -11775,7 +11859,7 @@
       <c r="A27" s="312" t="inlineStr"/>
       <c r="B27" s="312" t="inlineStr">
         <is>
-          <t>raw,16 频带</t>
+          <t>raw,d_model 64</t>
         </is>
       </c>
       <c r="C27" s="313" t="n"/>
@@ -11786,13 +11870,13 @@
       <c r="H27" s="313" t="n"/>
       <c r="I27" s="313" t="inlineStr">
         <is>
-          <t>0.3781±0.0467 (3)</t>
+          <t>0.3129±0.0121 (3)</t>
         </is>
       </c>
       <c r="J27" s="313" t="n"/>
       <c r="K27" s="313" t="inlineStr">
         <is>
-          <t>0.4288±0.0090 (3)</t>
+          <t>0.2780±0.0100 (3)</t>
         </is>
       </c>
       <c r="L27" s="313" t="n"/>
@@ -11801,7 +11885,7 @@
       <c r="A28" s="312" t="inlineStr"/>
       <c r="B28" s="312" t="inlineStr">
         <is>
-          <t>raw,patch_len 100</t>
+          <t>raw,d_model 256</t>
         </is>
       </c>
       <c r="C28" s="313" t="n"/>
@@ -11812,13 +11896,13 @@
       <c r="H28" s="313" t="n"/>
       <c r="I28" s="313" t="inlineStr">
         <is>
-          <t>0.3508±0.0251 (3)</t>
+          <t>0.4159±0.0529 (3)</t>
         </is>
       </c>
       <c r="J28" s="313" t="n"/>
       <c r="K28" s="313" t="inlineStr">
         <is>
-          <t>0.4066±0.0221 (3)</t>
+          <t>0.4437±0.0192 (3)</t>
         </is>
       </c>
       <c r="L28" s="313" t="n"/>
@@ -11827,7 +11911,7 @@
       <c r="A29" s="312" t="inlineStr"/>
       <c r="B29" s="312" t="inlineStr">
         <is>
-          <t>raw,dropout 0.5</t>
+          <t>raw,加宽</t>
         </is>
       </c>
       <c r="C29" s="313" t="n"/>
@@ -11838,13 +11922,13 @@
       <c r="H29" s="313" t="n"/>
       <c r="I29" s="313" t="inlineStr">
         <is>
-          <t>0.3409±0.0196 (3)</t>
+          <t>0.4093±0.0425 (3)</t>
         </is>
       </c>
       <c r="J29" s="313" t="n"/>
-      <c r="K29" s="313" t="inlineStr">
-        <is>
-          <t>0.4308±0.0139 (3)</t>
+      <c r="K29" s="315" t="inlineStr">
+        <is>
+          <t>0.4261±0.0085 (2)</t>
         </is>
       </c>
       <c r="L29" s="313" t="n"/>
@@ -11853,7 +11937,7 @@
       <c r="A30" s="312" t="inlineStr"/>
       <c r="B30" s="312" t="inlineStr">
         <is>
-          <t>raw,attn 头</t>
+          <t>raw,16 频带</t>
         </is>
       </c>
       <c r="C30" s="313" t="n"/>
@@ -11864,26 +11948,22 @@
       <c r="H30" s="313" t="n"/>
       <c r="I30" s="313" t="inlineStr">
         <is>
-          <t>0.3524±0.0467 (3)</t>
+          <t>0.3781±0.0467 (3)</t>
         </is>
       </c>
       <c r="J30" s="313" t="n"/>
       <c r="K30" s="313" t="inlineStr">
         <is>
-          <t>0.4545±0.0054 (3)</t>
+          <t>0.4288±0.0090 (3)</t>
         </is>
       </c>
       <c r="L30" s="313" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="311" t="inlineStr">
-        <is>
-          <t>已否决</t>
-        </is>
-      </c>
+      <c r="A31" s="312" t="inlineStr"/>
       <c r="B31" s="312" t="inlineStr">
         <is>
-          <t>spatial_pe: xyz(蒙太奇坐标)</t>
+          <t>raw,patch_len 100</t>
         </is>
       </c>
       <c r="C31" s="313" t="n"/>
@@ -11891,20 +11971,16 @@
       <c r="E31" s="313" t="n"/>
       <c r="F31" s="313" t="n"/>
       <c r="G31" s="313" t="n"/>
-      <c r="H31" s="313" t="inlineStr">
-        <is>
-          <t>0.6954±0.0167 (3)</t>
-        </is>
-      </c>
+      <c r="H31" s="313" t="n"/>
       <c r="I31" s="313" t="inlineStr">
         <is>
-          <t>0.2478±0.0053 (3)</t>
+          <t>0.3508±0.0251 (3)</t>
         </is>
       </c>
       <c r="J31" s="313" t="n"/>
       <c r="K31" s="313" t="inlineStr">
         <is>
-          <t>0.3338±0.0027 (3)</t>
+          <t>0.4066±0.0221 (3)</t>
         </is>
       </c>
       <c r="L31" s="313" t="n"/>
@@ -11913,7 +11989,7 @@
       <c r="A32" s="312" t="inlineStr"/>
       <c r="B32" s="312" t="inlineStr">
         <is>
-          <t>每窗口归一化</t>
+          <t>raw,dropout 0.5</t>
         </is>
       </c>
       <c r="C32" s="313" t="n"/>
@@ -11924,13 +12000,13 @@
       <c r="H32" s="313" t="n"/>
       <c r="I32" s="313" t="inlineStr">
         <is>
-          <t>0.2532±0.0155 (3)</t>
+          <t>0.3409±0.0196 (3)</t>
         </is>
       </c>
       <c r="J32" s="313" t="n"/>
       <c r="K32" s="313" t="inlineStr">
         <is>
-          <t>0.3050±0.0438 (3)</t>
+          <t>0.4308±0.0139 (3)</t>
         </is>
       </c>
       <c r="L32" s="313" t="n"/>
@@ -11939,7 +12015,7 @@
       <c r="A33" s="312" t="inlineStr"/>
       <c r="B33" s="312" t="inlineStr">
         <is>
-          <t>每窗口归一化 + raw</t>
+          <t>raw,attn 头</t>
         </is>
       </c>
       <c r="C33" s="313" t="n"/>
@@ -11948,24 +12024,28 @@
       <c r="F33" s="313" t="n"/>
       <c r="G33" s="313" t="n"/>
       <c r="H33" s="313" t="n"/>
-      <c r="I33" s="315" t="inlineStr">
-        <is>
-          <t>0.2896±0.0146 (2)</t>
+      <c r="I33" s="313" t="inlineStr">
+        <is>
+          <t>0.3524±0.0467 (3)</t>
         </is>
       </c>
       <c r="J33" s="313" t="n"/>
-      <c r="K33" s="315" t="inlineStr">
-        <is>
-          <t>0.2992±0.0139 (2)</t>
+      <c r="K33" s="313" t="inlineStr">
+        <is>
+          <t>0.4545±0.0054 (3)</t>
         </is>
       </c>
       <c r="L33" s="313" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="312" t="inlineStr"/>
+      <c r="A34" s="311" t="inlineStr">
+        <is>
+          <t>已否决</t>
+        </is>
+      </c>
       <c r="B34" s="312" t="inlineStr">
         <is>
-          <t>每受试者归一化</t>
+          <t>spatial_pe: xyz(蒙太奇坐标)</t>
         </is>
       </c>
       <c r="C34" s="313" t="n"/>
@@ -11973,21 +12053,29 @@
       <c r="E34" s="313" t="n"/>
       <c r="F34" s="313" t="n"/>
       <c r="G34" s="313" t="n"/>
-      <c r="H34" s="313" t="n"/>
-      <c r="I34" s="313" t="n"/>
-      <c r="J34" s="315" t="inlineStr">
-        <is>
-          <t>0.1328±0.0007 (2)</t>
-        </is>
-      </c>
-      <c r="K34" s="313" t="n"/>
+      <c r="H34" s="313" t="inlineStr">
+        <is>
+          <t>0.6954±0.0167 (3)</t>
+        </is>
+      </c>
+      <c r="I34" s="313" t="inlineStr">
+        <is>
+          <t>0.2478±0.0053 (3)</t>
+        </is>
+      </c>
+      <c r="J34" s="313" t="n"/>
+      <c r="K34" s="313" t="inlineStr">
+        <is>
+          <t>0.3338±0.0027 (3)</t>
+        </is>
+      </c>
       <c r="L34" s="313" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="312" t="inlineStr"/>
       <c r="B35" s="312" t="inlineStr">
         <is>
-          <t>每受试者归一化 + raw</t>
+          <t>每窗口归一化</t>
         </is>
       </c>
       <c r="C35" s="313" t="n"/>
@@ -11996,20 +12084,24 @@
       <c r="F35" s="313" t="n"/>
       <c r="G35" s="313" t="n"/>
       <c r="H35" s="313" t="n"/>
-      <c r="I35" s="313" t="n"/>
-      <c r="J35" s="313" t="inlineStr">
-        <is>
-          <t>0.1579±0.0034 (3)</t>
-        </is>
-      </c>
-      <c r="K35" s="313" t="n"/>
+      <c r="I35" s="313" t="inlineStr">
+        <is>
+          <t>0.2532±0.0155 (3)</t>
+        </is>
+      </c>
+      <c r="J35" s="313" t="n"/>
+      <c r="K35" s="313" t="inlineStr">
+        <is>
+          <t>0.3050±0.0438 (3)</t>
+        </is>
+      </c>
       <c r="L35" s="313" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="312" t="inlineStr"/>
       <c r="B36" s="312" t="inlineStr">
         <is>
-          <t>每受试者归一化 + raw + attn 头</t>
+          <t>每窗口归一化 + raw</t>
         </is>
       </c>
       <c r="C36" s="313" t="n"/>
@@ -12018,20 +12110,24 @@
       <c r="F36" s="313" t="n"/>
       <c r="G36" s="313" t="n"/>
       <c r="H36" s="313" t="n"/>
-      <c r="I36" s="313" t="n"/>
-      <c r="J36" s="313" t="inlineStr">
-        <is>
-          <t>0.1513±0.0012 (3)</t>
-        </is>
-      </c>
-      <c r="K36" s="313" t="n"/>
+      <c r="I36" s="315" t="inlineStr">
+        <is>
+          <t>0.2896±0.0146 (2)</t>
+        </is>
+      </c>
+      <c r="J36" s="313" t="n"/>
+      <c r="K36" s="315" t="inlineStr">
+        <is>
+          <t>0.2992±0.0139 (2)</t>
+        </is>
+      </c>
       <c r="L36" s="313" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="312" t="inlineStr"/>
       <c r="B37" s="312" t="inlineStr">
         <is>
-          <t>FACED 伪迹清洗</t>
+          <t>每受试者归一化</t>
         </is>
       </c>
       <c r="C37" s="313" t="n"/>
@@ -12041,9 +12137,9 @@
       <c r="G37" s="313" t="n"/>
       <c r="H37" s="313" t="n"/>
       <c r="I37" s="313" t="n"/>
-      <c r="J37" s="313" t="inlineStr">
-        <is>
-          <t>0.1346±0.0157 (3)</t>
+      <c r="J37" s="315" t="inlineStr">
+        <is>
+          <t>0.1328±0.0007 (2)</t>
         </is>
       </c>
       <c r="K37" s="313" t="n"/>
@@ -12053,7 +12149,7 @@
       <c r="A38" s="312" t="inlineStr"/>
       <c r="B38" s="312" t="inlineStr">
         <is>
-          <t>lr 1e-3</t>
+          <t>每受试者归一化 + raw</t>
         </is>
       </c>
       <c r="C38" s="313" t="n"/>
@@ -12062,24 +12158,20 @@
       <c r="F38" s="313" t="n"/>
       <c r="G38" s="313" t="n"/>
       <c r="H38" s="313" t="n"/>
-      <c r="I38" s="313" t="inlineStr">
-        <is>
-          <t>0.2498±0.0077 (3)</t>
-        </is>
-      </c>
-      <c r="J38" s="313" t="n"/>
-      <c r="K38" s="313" t="inlineStr">
-        <is>
-          <t>0.3094±0.0345 (3)</t>
-        </is>
-      </c>
+      <c r="I38" s="313" t="n"/>
+      <c r="J38" s="313" t="inlineStr">
+        <is>
+          <t>0.1579±0.0034 (3)</t>
+        </is>
+      </c>
+      <c r="K38" s="313" t="n"/>
       <c r="L38" s="313" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="312" t="inlineStr"/>
       <c r="B39" s="312" t="inlineStr">
         <is>
-          <t>lr 3e-4</t>
+          <t>每受试者归一化 + raw + attn 头</t>
         </is>
       </c>
       <c r="C39" s="313" t="n"/>
@@ -12088,42 +12180,34 @@
       <c r="F39" s="313" t="n"/>
       <c r="G39" s="313" t="n"/>
       <c r="H39" s="313" t="n"/>
-      <c r="I39" s="313" t="inlineStr">
-        <is>
-          <t>0.2623±0.0042 (3)</t>
-        </is>
-      </c>
-      <c r="J39" s="313" t="n"/>
-      <c r="K39" s="313" t="inlineStr">
-        <is>
-          <t>0.3495±0.0039 (3)</t>
-        </is>
-      </c>
+      <c r="I39" s="313" t="n"/>
+      <c r="J39" s="313" t="inlineStr">
+        <is>
+          <t>0.1513±0.0012 (3)</t>
+        </is>
+      </c>
+      <c r="K39" s="313" t="n"/>
       <c r="L39" s="313" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="311" t="inlineStr">
-        <is>
-          <t>早期 pilot</t>
-        </is>
-      </c>
+      <c r="A40" s="312" t="inlineStr"/>
       <c r="B40" s="312" t="inlineStr">
         <is>
-          <t>冻结前端 pilot</t>
+          <t>FACED 伪迹清洗</t>
         </is>
       </c>
       <c r="C40" s="313" t="n"/>
-      <c r="D40" s="313" t="inlineStr">
-        <is>
-          <t>0.6272±0.0099 (3)</t>
-        </is>
-      </c>
+      <c r="D40" s="313" t="n"/>
       <c r="E40" s="313" t="n"/>
       <c r="F40" s="313" t="n"/>
       <c r="G40" s="313" t="n"/>
       <c r="H40" s="313" t="n"/>
       <c r="I40" s="313" t="n"/>
-      <c r="J40" s="313" t="n"/>
+      <c r="J40" s="313" t="inlineStr">
+        <is>
+          <t>0.1346±0.0157 (3)</t>
+        </is>
+      </c>
       <c r="K40" s="313" t="n"/>
       <c r="L40" s="313" t="n"/>
     </row>
@@ -12131,112 +12215,190 @@
       <c r="A41" s="312" t="inlineStr"/>
       <c r="B41" s="312" t="inlineStr">
         <is>
-          <t>未滤波 pilot</t>
+          <t>lr 1e-3</t>
         </is>
       </c>
       <c r="C41" s="313" t="n"/>
-      <c r="D41" s="313" t="inlineStr">
-        <is>
-          <t>0.6209±0.0503 (3)</t>
-        </is>
-      </c>
+      <c r="D41" s="313" t="n"/>
       <c r="E41" s="313" t="n"/>
       <c r="F41" s="313" t="n"/>
       <c r="G41" s="313" t="n"/>
       <c r="H41" s="313" t="n"/>
-      <c r="I41" s="313" t="n"/>
+      <c r="I41" s="313" t="inlineStr">
+        <is>
+          <t>0.2498±0.0077 (3)</t>
+        </is>
+      </c>
       <c r="J41" s="313" t="n"/>
-      <c r="K41" s="313" t="n"/>
+      <c r="K41" s="313" t="inlineStr">
+        <is>
+          <t>0.3094±0.0345 (3)</t>
+        </is>
+      </c>
       <c r="L41" s="313" t="n"/>
     </row>
+    <row r="42">
+      <c r="A42" s="312" t="inlineStr"/>
+      <c r="B42" s="312" t="inlineStr">
+        <is>
+          <t>lr 3e-4</t>
+        </is>
+      </c>
+      <c r="C42" s="313" t="n"/>
+      <c r="D42" s="313" t="n"/>
+      <c r="E42" s="313" t="n"/>
+      <c r="F42" s="313" t="n"/>
+      <c r="G42" s="313" t="n"/>
+      <c r="H42" s="313" t="n"/>
+      <c r="I42" s="313" t="inlineStr">
+        <is>
+          <t>0.2623±0.0042 (3)</t>
+        </is>
+      </c>
+      <c r="J42" s="313" t="n"/>
+      <c r="K42" s="313" t="inlineStr">
+        <is>
+          <t>0.3495±0.0039 (3)</t>
+        </is>
+      </c>
+      <c r="L42" s="313" t="n"/>
+    </row>
     <row r="43">
-      <c r="A43" s="316" t="inlineStr">
+      <c r="A43" s="311" t="inlineStr">
+        <is>
+          <t>早期 pilot</t>
+        </is>
+      </c>
+      <c r="B43" s="312" t="inlineStr">
+        <is>
+          <t>冻结前端 pilot</t>
+        </is>
+      </c>
+      <c r="C43" s="313" t="n"/>
+      <c r="D43" s="313" t="inlineStr">
+        <is>
+          <t>0.6272±0.0099 (3)</t>
+        </is>
+      </c>
+      <c r="E43" s="313" t="n"/>
+      <c r="F43" s="313" t="n"/>
+      <c r="G43" s="313" t="n"/>
+      <c r="H43" s="313" t="n"/>
+      <c r="I43" s="313" t="n"/>
+      <c r="J43" s="313" t="n"/>
+      <c r="K43" s="313" t="n"/>
+      <c r="L43" s="313" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="312" t="inlineStr"/>
+      <c r="B44" s="312" t="inlineStr">
+        <is>
+          <t>未滤波 pilot</t>
+        </is>
+      </c>
+      <c r="C44" s="313" t="n"/>
+      <c r="D44" s="313" t="inlineStr">
+        <is>
+          <t>0.6209±0.0503 (3)</t>
+        </is>
+      </c>
+      <c r="E44" s="313" t="n"/>
+      <c r="F44" s="313" t="n"/>
+      <c r="G44" s="313" t="n"/>
+      <c r="H44" s="313" t="n"/>
+      <c r="I44" s="313" t="n"/>
+      <c r="J44" s="313" t="n"/>
+      <c r="K44" s="313" t="n"/>
+      <c r="L44" s="313" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="316" t="inlineStr">
         <is>
           <t>样本量消融</t>
         </is>
       </c>
-      <c r="B43" s="317" t="inlineStr">
+      <c r="B46" s="317" t="inlineStr">
         <is>
           <t>TUEV 训练集降采样(kappa) —— 检验等级三是否只是样本量问题</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="309" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="309" t="inlineStr">
         <is>
           <t>模型</t>
         </is>
       </c>
-      <c r="C44" s="310" t="inlineStr">
+      <c r="C47" s="310" t="inlineStr">
         <is>
           <t>n=2160</t>
         </is>
       </c>
-      <c r="D44" s="310" t="inlineStr">
+      <c r="D47" s="310" t="inlineStr">
         <is>
           <t>n=6720</t>
         </is>
       </c>
-      <c r="E44" s="310" t="inlineStr">
+      <c r="E47" s="310" t="inlineStr">
         <is>
           <t>n=20000</t>
         </is>
       </c>
-      <c r="F44" s="310" t="inlineStr">
+      <c r="F47" s="310" t="inlineStr">
         <is>
           <t>全量 68445</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" s="312" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="312" t="inlineStr">
         <is>
           <t>PACLock v2</t>
         </is>
       </c>
-      <c r="C45" s="315" t="inlineStr">
+      <c r="C48" s="315" t="inlineStr">
         <is>
           <t>0.6523±0.0000 (1)</t>
         </is>
       </c>
-      <c r="D45" s="315" t="inlineStr">
+      <c r="D48" s="315" t="inlineStr">
         <is>
           <t>0.7098±0.0000 (1)</t>
         </is>
       </c>
-      <c r="E45" s="315" t="inlineStr">
+      <c r="E48" s="315" t="inlineStr">
         <is>
           <t>0.6767±0.0000 (1)</t>
         </is>
       </c>
-      <c r="F45" s="313" t="inlineStr">
+      <c r="F48" s="313" t="inlineStr">
         <is>
           <t>0.7076±0.0311 (3)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="312" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="312" t="inlineStr">
         <is>
           <t>SPaRCNet</t>
         </is>
       </c>
-      <c r="C46" s="315" t="inlineStr">
+      <c r="C49" s="315" t="inlineStr">
         <is>
           <t>0.4917±0.0000 (1)</t>
         </is>
       </c>
-      <c r="D46" s="315" t="inlineStr">
+      <c r="D49" s="315" t="inlineStr">
         <is>
           <t>0.5532±0.0000 (1)</t>
         </is>
       </c>
-      <c r="E46" s="315" t="inlineStr">
+      <c r="E49" s="315" t="inlineStr">
         <is>
           <t>0.3642±0.0000 (1)</t>
         </is>
       </c>
-      <c r="F46" s="313" t="inlineStr">
+      <c r="F49" s="313" t="inlineStr">
         <is>
           <t>0.4885±0.0279 (3)</t>
         </is>
@@ -12256,7 +12418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="219" min="1" max="4"/>
@@ -12995,15 +13157,41 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="220"/>
-    <row r="22" ht="13.75" customHeight="1" s="220">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="220">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="318" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="319" t="n"/>
+      <c r="D21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="319" t="n"/>
+      <c r="H21" s="299" t="n"/>
+      <c r="I21" s="299" t="n"/>
+    </row>
+    <row r="22" ht="13.75" customHeight="1" s="220"/>
+    <row r="23" ht="15" customHeight="1" s="220">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="220"/>
     <row r="24" ht="15" customHeight="1" s="220"/>
     <row r="25" ht="15" customHeight="1" s="220"/>
     <row r="26" ht="15" customHeight="1" s="220"/>
@@ -13061,7 +13249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="219" min="1" max="4"/>
@@ -13824,15 +14012,55 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="220"/>
-    <row r="22" ht="13.75" customHeight="1" s="220">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="220">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="318" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="319" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="D21" s="320" t="inlineStr">
+        <is>
+          <t>0.6410 (1 seed)</t>
+        </is>
+      </c>
+      <c r="E21" s="320" t="inlineStr">
+        <is>
+          <t>0.6951 (1 seed)</t>
+        </is>
+      </c>
+      <c r="F21" s="320" t="inlineStr">
+        <is>
+          <t>0.8365 (1 seed)</t>
+        </is>
+      </c>
+      <c r="G21" s="320" t="inlineStr">
+        <is>
+          <t>-0.0125</t>
+        </is>
+      </c>
+      <c r="H21" s="321" t="inlineStr">
+        <is>
+          <t>+0.0221</t>
+        </is>
+      </c>
+      <c r="I21" s="321" t="inlineStr">
+        <is>
+          <t>+0.0428</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="13.75" customHeight="1" s="220"/>
+    <row r="23" ht="15" customHeight="1" s="220">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="220"/>
     <row r="24" ht="15" customHeight="1" s="220"/>
     <row r="25" ht="15" customHeight="1" s="220"/>
     <row r="26" ht="15" customHeight="1" s="220"/>
@@ -13891,7 +14119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="219" min="1" max="4"/>
@@ -14654,15 +14882,55 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="220"/>
-    <row r="22" ht="13.55" customHeight="1" s="220">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="220">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="318" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="319" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="D21" s="320" t="inlineStr">
+        <is>
+          <t>0.5901 (1 seed)</t>
+        </is>
+      </c>
+      <c r="E21" s="320" t="inlineStr">
+        <is>
+          <t>0.6299 (1 seed)</t>
+        </is>
+      </c>
+      <c r="F21" s="320" t="inlineStr">
+        <is>
+          <t>0.9276 (1 seed)</t>
+        </is>
+      </c>
+      <c r="G21" s="320" t="inlineStr">
+        <is>
+          <t>+0.0417</t>
+        </is>
+      </c>
+      <c r="H21" s="321" t="inlineStr">
+        <is>
+          <t>-0.0099</t>
+        </is>
+      </c>
+      <c r="I21" s="321" t="inlineStr">
+        <is>
+          <t>+0.0010</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="13.55" customHeight="1" s="220"/>
+    <row r="23" ht="15" customHeight="1" s="220">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="220"/>
     <row r="24" ht="15" customHeight="1" s="220"/>
     <row r="25" ht="13.55" customHeight="1" s="220"/>
     <row r="26" ht="13.55" customHeight="1" s="220"/>
@@ -14718,7 +14986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="219" min="1" max="4"/>
@@ -15481,15 +15749,55 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="220"/>
-    <row r="22" ht="13.75" customHeight="1" s="220">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="220">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="318" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="319" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="D21" s="320" t="inlineStr">
+        <is>
+          <t>0.5290 (1 seed)</t>
+        </is>
+      </c>
+      <c r="E21" s="320" t="inlineStr">
+        <is>
+          <t>0.7473 (1 seed)</t>
+        </is>
+      </c>
+      <c r="F21" s="320" t="inlineStr">
+        <is>
+          <t>0.9368 (1 seed)</t>
+        </is>
+      </c>
+      <c r="G21" s="320" t="inlineStr">
+        <is>
+          <t>+0.2009</t>
+        </is>
+      </c>
+      <c r="H21" s="321" t="inlineStr">
+        <is>
+          <t>+0.0643</t>
+        </is>
+      </c>
+      <c r="I21" s="321" t="inlineStr">
+        <is>
+          <t>+0.1311</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="13.75" customHeight="1" s="220"/>
+    <row r="23" ht="15" customHeight="1" s="220">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="220"/>
     <row r="24" ht="15" customHeight="1" s="220"/>
     <row r="25" ht="15" customHeight="1" s="220"/>
     <row r="26" ht="15" customHeight="1" s="220"/>
@@ -15546,7 +15854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="219" min="1" max="4"/>
@@ -16309,15 +16617,41 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="220"/>
-    <row r="22" ht="13.55" customHeight="1" s="220">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="220">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="318" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="319" t="n"/>
+      <c r="D21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="319" t="n"/>
+      <c r="H21" s="299" t="n"/>
+      <c r="I21" s="299" t="n"/>
+    </row>
+    <row r="22" ht="13.55" customHeight="1" s="220"/>
+    <row r="23" ht="15" customHeight="1" s="220">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="220"/>
     <row r="24" ht="15" customHeight="1" s="220"/>
     <row r="25" ht="13.55" customHeight="1" s="220"/>
     <row r="26" ht="13.55" customHeight="1" s="220"/>
@@ -16377,7 +16711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66667" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="219" min="1" max="4"/>
@@ -17140,15 +17474,41 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="220"/>
-    <row r="22" ht="13.55" customHeight="1" s="220">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="220">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="318" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="319" t="n"/>
+      <c r="D21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="319" t="n"/>
+      <c r="H21" s="299" t="n"/>
+      <c r="I21" s="299" t="n"/>
+    </row>
+    <row r="22" ht="13.55" customHeight="1" s="220"/>
+    <row r="23" ht="15" customHeight="1" s="220">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="220"/>
     <row r="24" ht="15" customHeight="1" s="220"/>
     <row r="25" ht="13.55" customHeight="1" s="220"/>
     <row r="26" ht="13.55" customHeight="1" s="220"/>
@@ -17203,7 +17563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="219" min="1" max="4"/>
@@ -17966,15 +18326,41 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="123.8" customHeight="1" s="220"/>
-    <row r="22" ht="13.55" customHeight="1" s="220">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21" ht="123.8" customHeight="1" s="220">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="318" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="319" t="n"/>
+      <c r="D21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="319" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="299" t="n"/>
+      <c r="H21" s="299" t="n"/>
+      <c r="I21" s="299" t="n"/>
+    </row>
+    <row r="22" ht="13.55" customHeight="1" s="220"/>
+    <row r="23" ht="13.55" customHeight="1" s="220">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="13.55" customHeight="1" s="220"/>
     <row r="24" ht="13.55" customHeight="1" s="220"/>
     <row r="25" ht="13.55" customHeight="1" s="220"/>
     <row r="26" ht="13.55" customHeight="1" s="220"/>
@@ -18032,7 +18418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="220" min="1" max="1"/>
@@ -18762,8 +19148,35 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="300" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="297" t="n"/>
+      <c r="B21" s="298" t="inlineStr">
+        <is>
+          <t>PACLock (hybrid)</t>
+        </is>
+      </c>
+      <c r="C21" s="299" t="n"/>
+      <c r="D21" s="299" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="299" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="299" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="299" t="n"/>
+      <c r="H21" s="299" t="n"/>
+      <c r="I21" s="299" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="300" t="inlineStr">
         <is>
           <t>灰色行 = 该 baseline 的原论文未评测本数据集,不存在官方超参;所用配方由我们从该模型覆盖过的数据集迁移而来。这些数字反映的是「该架构在我们所选配方下的表现」,不是「该 baseline 已发表的能力」。</t>
         </is>

</xml_diff>

<commit_message>
xlsx: rung-0 complete -- CHB-MIT hybrid+gate 0.7513 is the project best
The ablation sheet now carries the finished rung-0 sweep (135 cells). CHB-MIT
hybrid+gate lands at 0.7513 (1 seed), above plain hybrid 0.7473, raw 0.6672,
and the best external baseline by +0.124. The gate is now positive on CHB-MIT
as well as TUSZ/BCI, negative nowhere tested -- the leading configuration is
hybrid + mean head + per-band gate.

Rung-0 verdict as it stands, all hybrid cells single-seed: two wins (CHB-MIT
decisively, TUEV over raw but not over pure rotation), two losses to raw by
0.02-0.03 (TUSZ, BCI). The design goal of >= raw everywhere is NOT met.

The CHB-MIT transplant arms both landed at an identical 0.5079 -- a degenerate
tie on a host that is weak there anyway (CBraMod scratch 0.3169) -- and are
treated as void, entering no table.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/PACLock_baseline_matrix_filled.xlsx
+++ b/results/PACLock_baseline_matrix_filled.xlsx
@@ -11359,7 +11359,11 @@
           <t>0.6455±0.0000 (1)</t>
         </is>
       </c>
-      <c r="F12" s="313" t="n"/>
+      <c r="F12" s="315" t="inlineStr">
+        <is>
+          <t>0.7513±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="G12" s="313" t="n"/>
       <c r="H12" s="313" t="n"/>
       <c r="I12" s="313" t="n"/>

</xml_diff>

<commit_message>
xlsx: hybrid+spatial rows -- the middle-zone verdict on the MI corpora
hybrid+spatial lands between pac+spatial and raw+spatial on both MI corpora,
same direction twice: BCI 0.4888 / gated 0.4923 against raw+spatial 0.5274;
PhysioNet-MI 0.4284 / 0.4258 against 0.4840. All single seed. The right head
recovers most of what the mean head lost (BCI 0.391 -> 0.492) and clears
pac+spatial by a wide margin, but the interaction rows still carry a real net
cost on motor imagery -- the gate moves +-0.003 and does not close it.

Standing picture per corpus, best of ours: CHB-MIT hybrid+gate 0.7513; TUEV
rotation 0.7328(3); TUSZ rotation 0.6884(1); BCI and PhysioNet-MI raw+spatial
0.5274(1)/0.4840(1). Hybrid is the CHB-MIT champion, not the universal form.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/PACLock_baseline_matrix_filled.xlsx
+++ b/results/PACLock_baseline_matrix_filled.xlsx
@@ -10966,7 +10966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="220" min="1" max="1"/>
@@ -11413,52 +11413,24 @@
       <c r="A14" s="312" t="inlineStr"/>
       <c r="B14" s="312" t="inlineStr">
         <is>
-          <t>rotation(耦合只旋转不缩放)</t>
-        </is>
-      </c>
-      <c r="C14" s="315" t="inlineStr">
-        <is>
-          <t>0.8806±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="D14" s="313" t="inlineStr">
-        <is>
-          <t>0.7328±0.0161 (3)</t>
-        </is>
-      </c>
-      <c r="E14" s="315" t="inlineStr">
-        <is>
-          <t>0.6884±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="F14" s="315" t="inlineStr">
-        <is>
-          <t>0.5100±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="G14" s="315" t="inlineStr">
-        <is>
-          <t>0.6449±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="H14" s="315" t="inlineStr">
-        <is>
-          <t>0.7104±0.0000 (1)</t>
-        </is>
-      </c>
+          <t>hybrid + spatial 头</t>
+        </is>
+      </c>
+      <c r="C14" s="313" t="n"/>
+      <c r="D14" s="313" t="n"/>
+      <c r="E14" s="313" t="n"/>
+      <c r="F14" s="313" t="n"/>
+      <c r="G14" s="313" t="n"/>
+      <c r="H14" s="313" t="n"/>
       <c r="I14" s="315" t="inlineStr">
         <is>
-          <t>0.2916±0.0063 (2)</t>
-        </is>
-      </c>
-      <c r="J14" s="315" t="inlineStr">
-        <is>
-          <t>0.1514±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="K14" s="313" t="inlineStr">
-        <is>
-          <t>0.3708±0.0092 (3)</t>
+          <t>0.4284±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J14" s="313" t="n"/>
+      <c r="K14" s="315" t="inlineStr">
+        <is>
+          <t>0.4888±0.0000 (1)</t>
         </is>
       </c>
       <c r="L14" s="313" t="n"/>
@@ -11467,7 +11439,7 @@
       <c r="A15" s="312" t="inlineStr"/>
       <c r="B15" s="312" t="inlineStr">
         <is>
-          <t>rotation(跑在 PAC 协议数据上,与上行不可比)</t>
+          <t>hybrid + spatial 头 + 门</t>
         </is>
       </c>
       <c r="C15" s="313" t="n"/>
@@ -11476,43 +11448,59 @@
       <c r="F15" s="313" t="n"/>
       <c r="G15" s="313" t="n"/>
       <c r="H15" s="313" t="n"/>
-      <c r="I15" s="313" t="n"/>
-      <c r="J15" s="315" t="inlineStr">
-        <is>
-          <t>0.1098±0.0000 (1)</t>
-        </is>
-      </c>
+      <c r="I15" s="315" t="inlineStr">
+        <is>
+          <t>0.4258±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J15" s="313" t="n"/>
       <c r="K15" s="315" t="inlineStr">
         <is>
-          <t>0.2724±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="L15" s="315" t="inlineStr">
-        <is>
-          <t>0.5568±0.0000 (1)</t>
-        </is>
-      </c>
+          <t>0.4923±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="L15" s="313" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="312" t="inlineStr"/>
       <c r="B16" s="312" t="inlineStr">
         <is>
-          <t>spatial 头(保留电极身份)</t>
-        </is>
-      </c>
-      <c r="C16" s="313" t="n"/>
-      <c r="D16" s="315" t="inlineStr">
-        <is>
-          <t>0.6520±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="E16" s="313" t="n"/>
-      <c r="F16" s="313" t="n"/>
-      <c r="G16" s="313" t="n"/>
-      <c r="H16" s="313" t="n"/>
-      <c r="I16" s="313" t="inlineStr">
-        <is>
-          <t>0.3535±0.0047 (3)</t>
+          <t>rotation(耦合只旋转不缩放)</t>
+        </is>
+      </c>
+      <c r="C16" s="315" t="inlineStr">
+        <is>
+          <t>0.8806±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="D16" s="313" t="inlineStr">
+        <is>
+          <t>0.7328±0.0161 (3)</t>
+        </is>
+      </c>
+      <c r="E16" s="315" t="inlineStr">
+        <is>
+          <t>0.6884±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="F16" s="315" t="inlineStr">
+        <is>
+          <t>0.5100±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="G16" s="315" t="inlineStr">
+        <is>
+          <t>0.6449±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="H16" s="315" t="inlineStr">
+        <is>
+          <t>0.7104±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="I16" s="315" t="inlineStr">
+        <is>
+          <t>0.2916±0.0063 (2)</t>
         </is>
       </c>
       <c r="J16" s="315" t="inlineStr">
@@ -11522,7 +11510,7 @@
       </c>
       <c r="K16" s="313" t="inlineStr">
         <is>
-          <t>0.4317±0.0153 (3)</t>
+          <t>0.3708±0.0092 (3)</t>
         </is>
       </c>
       <c r="L16" s="313" t="n"/>
@@ -11531,7 +11519,7 @@
       <c r="A17" s="312" t="inlineStr"/>
       <c r="B17" s="312" t="inlineStr">
         <is>
-          <t>rotation + spatial 头</t>
+          <t>rotation(跑在 PAC 协议数据上,与上行不可比)</t>
         </is>
       </c>
       <c r="C17" s="313" t="n"/>
@@ -11540,73 +11528,53 @@
       <c r="F17" s="313" t="n"/>
       <c r="G17" s="313" t="n"/>
       <c r="H17" s="313" t="n"/>
-      <c r="I17" s="315" t="inlineStr">
-        <is>
-          <t>0.3299±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="J17" s="313" t="n"/>
+      <c r="I17" s="313" t="n"/>
+      <c r="J17" s="315" t="inlineStr">
+        <is>
+          <t>0.1098±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="K17" s="315" t="inlineStr">
         <is>
-          <t>0.4344±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="L17" s="313" t="n"/>
+          <t>0.2724±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="L17" s="315" t="inlineStr">
+        <is>
+          <t>0.5568±0.0000 (1)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="311" t="inlineStr">
-        <is>
-          <t>预训练</t>
-        </is>
-      </c>
+      <c r="A18" s="312" t="inlineStr"/>
       <c r="B18" s="312" t="inlineStr">
         <is>
-          <t>预训练 base(60k)</t>
-        </is>
-      </c>
-      <c r="C18" s="313" t="inlineStr">
-        <is>
-          <t>0.8841±0.0043 (3)</t>
-        </is>
-      </c>
-      <c r="D18" s="313" t="inlineStr">
-        <is>
-          <t>0.6730±0.0116 (3)</t>
-        </is>
-      </c>
-      <c r="E18" s="313" t="inlineStr">
-        <is>
-          <t>0.6398±0.0615 (3)</t>
-        </is>
-      </c>
-      <c r="F18" s="313" t="inlineStr">
-        <is>
-          <t>0.6830±0.0228 (3)</t>
-        </is>
-      </c>
-      <c r="G18" s="313" t="inlineStr">
-        <is>
-          <t>0.6651±0.0109 (3)</t>
-        </is>
-      </c>
-      <c r="H18" s="313" t="inlineStr">
-        <is>
-          <t>0.6934±0.0032 (3)</t>
-        </is>
-      </c>
+          <t>spatial 头(保留电极身份)</t>
+        </is>
+      </c>
+      <c r="C18" s="313" t="n"/>
+      <c r="D18" s="315" t="inlineStr">
+        <is>
+          <t>0.6520±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="E18" s="313" t="n"/>
+      <c r="F18" s="313" t="n"/>
+      <c r="G18" s="313" t="n"/>
+      <c r="H18" s="313" t="n"/>
       <c r="I18" s="313" t="inlineStr">
         <is>
-          <t>0.3059±0.0262 (3)</t>
-        </is>
-      </c>
-      <c r="J18" s="313" t="inlineStr">
-        <is>
-          <t>0.1540±0.0202 (3)</t>
+          <t>0.3535±0.0047 (3)</t>
+        </is>
+      </c>
+      <c r="J18" s="315" t="inlineStr">
+        <is>
+          <t>0.1514±0.0000 (1)</t>
         </is>
       </c>
       <c r="K18" s="313" t="inlineStr">
         <is>
-          <t>0.3652±0.0083 (3)</t>
+          <t>0.4317±0.0153 (3)</t>
         </is>
       </c>
       <c r="L18" s="313" t="n"/>
@@ -11615,90 +11583,82 @@
       <c r="A19" s="312" t="inlineStr"/>
       <c r="B19" s="312" t="inlineStr">
         <is>
-          <t>预训练 large(60k)</t>
-        </is>
-      </c>
-      <c r="C19" s="313" t="inlineStr">
-        <is>
-          <t>0.8869±0.0069 (3)</t>
-        </is>
-      </c>
-      <c r="D19" s="313" t="inlineStr">
-        <is>
-          <t>0.6523±0.0302 (3)</t>
-        </is>
-      </c>
-      <c r="E19" s="313" t="inlineStr">
-        <is>
-          <t>0.6289±0.0297 (3)</t>
-        </is>
-      </c>
-      <c r="F19" s="313" t="inlineStr">
-        <is>
-          <t>0.6162±0.0467 (3)</t>
-        </is>
-      </c>
-      <c r="G19" s="313" t="inlineStr">
-        <is>
-          <t>0.6641±0.0044 (3)</t>
-        </is>
-      </c>
-      <c r="H19" s="313" t="inlineStr">
-        <is>
-          <t>0.6996±0.0153 (3)</t>
-        </is>
-      </c>
-      <c r="I19" s="313" t="inlineStr">
-        <is>
-          <t>0.3140±0.0094 (3)</t>
-        </is>
-      </c>
-      <c r="J19" s="313" t="inlineStr">
-        <is>
-          <t>0.1640±0.0155 (3)</t>
-        </is>
-      </c>
-      <c r="K19" s="313" t="inlineStr">
-        <is>
-          <t>0.4122±0.0166 (3)</t>
+          <t>rotation + spatial 头</t>
+        </is>
+      </c>
+      <c r="C19" s="313" t="n"/>
+      <c r="D19" s="313" t="n"/>
+      <c r="E19" s="313" t="n"/>
+      <c r="F19" s="313" t="n"/>
+      <c r="G19" s="313" t="n"/>
+      <c r="H19" s="313" t="n"/>
+      <c r="I19" s="315" t="inlineStr">
+        <is>
+          <t>0.3299±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J19" s="313" t="n"/>
+      <c r="K19" s="315" t="inlineStr">
+        <is>
+          <t>0.4344±0.0000 (1)</t>
         </is>
       </c>
       <c r="L19" s="313" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="312" t="inlineStr"/>
+      <c r="A20" s="311" t="inlineStr">
+        <is>
+          <t>预训练</t>
+        </is>
+      </c>
       <c r="B20" s="312" t="inlineStr">
         <is>
-          <t>raw tokenizer 预训练 large(60k)</t>
-        </is>
-      </c>
-      <c r="C20" s="313" t="n"/>
-      <c r="D20" s="313" t="n"/>
-      <c r="E20" s="315" t="inlineStr">
-        <is>
-          <t>0.5460±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="F20" s="315" t="inlineStr">
-        <is>
-          <t>0.6279±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="G20" s="313" t="n"/>
-      <c r="H20" s="313" t="n"/>
+          <t>预训练 base(60k)</t>
+        </is>
+      </c>
+      <c r="C20" s="313" t="inlineStr">
+        <is>
+          <t>0.8841±0.0043 (3)</t>
+        </is>
+      </c>
+      <c r="D20" s="313" t="inlineStr">
+        <is>
+          <t>0.6730±0.0116 (3)</t>
+        </is>
+      </c>
+      <c r="E20" s="313" t="inlineStr">
+        <is>
+          <t>0.6398±0.0615 (3)</t>
+        </is>
+      </c>
+      <c r="F20" s="313" t="inlineStr">
+        <is>
+          <t>0.6830±0.0228 (3)</t>
+        </is>
+      </c>
+      <c r="G20" s="313" t="inlineStr">
+        <is>
+          <t>0.6651±0.0109 (3)</t>
+        </is>
+      </c>
+      <c r="H20" s="313" t="inlineStr">
+        <is>
+          <t>0.6934±0.0032 (3)</t>
+        </is>
+      </c>
       <c r="I20" s="313" t="inlineStr">
         <is>
-          <t>0.3633±0.0349 (3)</t>
-        </is>
-      </c>
-      <c r="J20" s="315" t="inlineStr">
-        <is>
-          <t>0.1690±0.0018 (2)</t>
+          <t>0.3059±0.0262 (3)</t>
+        </is>
+      </c>
+      <c r="J20" s="313" t="inlineStr">
+        <is>
+          <t>0.1540±0.0202 (3)</t>
         </is>
       </c>
       <c r="K20" s="313" t="inlineStr">
         <is>
-          <t>0.4483±0.0031 (3)</t>
+          <t>0.3652±0.0083 (3)</t>
         </is>
       </c>
       <c r="L20" s="313" t="n"/>
@@ -11707,73 +11667,117 @@
       <c r="A21" s="312" t="inlineStr"/>
       <c r="B21" s="312" t="inlineStr">
         <is>
-          <t>预训练池剔除 TUSZ/CHB-MIT</t>
-        </is>
-      </c>
-      <c r="C21" s="313" t="n"/>
-      <c r="D21" s="313" t="n"/>
-      <c r="E21" s="315" t="inlineStr">
-        <is>
-          <t>0.6221±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="F21" s="315" t="inlineStr">
-        <is>
-          <t>0.6410±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="G21" s="313" t="n"/>
-      <c r="H21" s="313" t="n"/>
-      <c r="I21" s="313" t="n"/>
-      <c r="J21" s="313" t="n"/>
-      <c r="K21" s="313" t="n"/>
+          <t>预训练 large(60k)</t>
+        </is>
+      </c>
+      <c r="C21" s="313" t="inlineStr">
+        <is>
+          <t>0.8869±0.0069 (3)</t>
+        </is>
+      </c>
+      <c r="D21" s="313" t="inlineStr">
+        <is>
+          <t>0.6523±0.0302 (3)</t>
+        </is>
+      </c>
+      <c r="E21" s="313" t="inlineStr">
+        <is>
+          <t>0.6289±0.0297 (3)</t>
+        </is>
+      </c>
+      <c r="F21" s="313" t="inlineStr">
+        <is>
+          <t>0.6162±0.0467 (3)</t>
+        </is>
+      </c>
+      <c r="G21" s="313" t="inlineStr">
+        <is>
+          <t>0.6641±0.0044 (3)</t>
+        </is>
+      </c>
+      <c r="H21" s="313" t="inlineStr">
+        <is>
+          <t>0.6996±0.0153 (3)</t>
+        </is>
+      </c>
+      <c r="I21" s="313" t="inlineStr">
+        <is>
+          <t>0.3140±0.0094 (3)</t>
+        </is>
+      </c>
+      <c r="J21" s="313" t="inlineStr">
+        <is>
+          <t>0.1640±0.0155 (3)</t>
+        </is>
+      </c>
+      <c r="K21" s="313" t="inlineStr">
+        <is>
+          <t>0.4122±0.0166 (3)</t>
+        </is>
+      </c>
       <c r="L21" s="313" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="312" t="inlineStr"/>
       <c r="B22" s="312" t="inlineStr">
         <is>
-          <t>预训练 base,微调 patch_len=200</t>
+          <t>raw tokenizer 预训练 large(60k)</t>
         </is>
       </c>
       <c r="C22" s="313" t="n"/>
-      <c r="D22" s="313" t="inlineStr">
-        <is>
-          <t>0.6793±0.0109 (3)</t>
-        </is>
-      </c>
-      <c r="E22" s="313" t="n"/>
-      <c r="F22" s="313" t="n"/>
+      <c r="D22" s="313" t="n"/>
+      <c r="E22" s="315" t="inlineStr">
+        <is>
+          <t>0.5460±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="F22" s="315" t="inlineStr">
+        <is>
+          <t>0.6279±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="G22" s="313" t="n"/>
       <c r="H22" s="313" t="n"/>
-      <c r="I22" s="313" t="n"/>
-      <c r="J22" s="313" t="n"/>
-      <c r="K22" s="313" t="n"/>
+      <c r="I22" s="313" t="inlineStr">
+        <is>
+          <t>0.3633±0.0349 (3)</t>
+        </is>
+      </c>
+      <c r="J22" s="315" t="inlineStr">
+        <is>
+          <t>0.1690±0.0018 (2)</t>
+        </is>
+      </c>
+      <c r="K22" s="313" t="inlineStr">
+        <is>
+          <t>0.4483±0.0031 (3)</t>
+        </is>
+      </c>
       <c r="L22" s="313" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="312" t="inlineStr"/>
       <c r="B23" s="312" t="inlineStr">
         <is>
-          <t>早期微调配方(6k checkpoint)</t>
+          <t>预训练池剔除 TUSZ/CHB-MIT</t>
         </is>
       </c>
       <c r="C23" s="313" t="n"/>
       <c r="D23" s="313" t="n"/>
-      <c r="E23" s="313" t="n"/>
-      <c r="F23" s="313" t="n"/>
+      <c r="E23" s="315" t="inlineStr">
+        <is>
+          <t>0.6221±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="F23" s="315" t="inlineStr">
+        <is>
+          <t>0.6410±0.0000 (1)</t>
+        </is>
+      </c>
       <c r="G23" s="313" t="n"/>
       <c r="H23" s="313" t="n"/>
-      <c r="I23" s="315" t="inlineStr">
-        <is>
-          <t>0.2690±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="J23" s="315" t="inlineStr">
-        <is>
-          <t>0.1279±0.0000 (1)</t>
-        </is>
-      </c>
+      <c r="I23" s="313" t="n"/>
+      <c r="J23" s="313" t="n"/>
       <c r="K23" s="313" t="n"/>
       <c r="L23" s="313" t="n"/>
     </row>
@@ -11781,25 +11785,21 @@
       <c r="A24" s="312" t="inlineStr"/>
       <c r="B24" s="312" t="inlineStr">
         <is>
-          <t>早期微调配方 v2(6k checkpoint)</t>
+          <t>预训练 base,微调 patch_len=200</t>
         </is>
       </c>
       <c r="C24" s="313" t="n"/>
-      <c r="D24" s="313" t="n"/>
+      <c r="D24" s="313" t="inlineStr">
+        <is>
+          <t>0.6793±0.0109 (3)</t>
+        </is>
+      </c>
       <c r="E24" s="313" t="n"/>
       <c r="F24" s="313" t="n"/>
       <c r="G24" s="313" t="n"/>
       <c r="H24" s="313" t="n"/>
-      <c r="I24" s="315" t="inlineStr">
-        <is>
-          <t>0.2622±0.0000 (1)</t>
-        </is>
-      </c>
-      <c r="J24" s="315" t="inlineStr">
-        <is>
-          <t>0.1408±0.0000 (1)</t>
-        </is>
-      </c>
+      <c r="I24" s="313" t="n"/>
+      <c r="J24" s="313" t="n"/>
       <c r="K24" s="313" t="n"/>
       <c r="L24" s="313" t="n"/>
     </row>
@@ -11807,7 +11807,7 @@
       <c r="A25" s="312" t="inlineStr"/>
       <c r="B25" s="312" t="inlineStr">
         <is>
-          <t>早期微调配方 large(6k checkpoint)</t>
+          <t>早期微调配方(6k checkpoint)</t>
         </is>
       </c>
       <c r="C25" s="313" t="n"/>
@@ -11818,26 +11818,22 @@
       <c r="H25" s="313" t="n"/>
       <c r="I25" s="315" t="inlineStr">
         <is>
-          <t>0.2716±0.0000 (1)</t>
+          <t>0.2690±0.0000 (1)</t>
         </is>
       </c>
       <c r="J25" s="315" t="inlineStr">
         <is>
-          <t>0.1381±0.0000 (1)</t>
+          <t>0.1279±0.0000 (1)</t>
         </is>
       </c>
       <c r="K25" s="313" t="n"/>
       <c r="L25" s="313" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="311" t="inlineStr">
-        <is>
-          <t>容量阶梯</t>
-        </is>
-      </c>
+      <c r="A26" s="312" t="inlineStr"/>
       <c r="B26" s="312" t="inlineStr">
         <is>
-          <t>raw,d_model 32</t>
+          <t>早期微调配方 v2(6k checkpoint)</t>
         </is>
       </c>
       <c r="C26" s="313" t="n"/>
@@ -11846,24 +11842,24 @@
       <c r="F26" s="313" t="n"/>
       <c r="G26" s="313" t="n"/>
       <c r="H26" s="313" t="n"/>
-      <c r="I26" s="313" t="inlineStr">
-        <is>
-          <t>0.2613±0.0100 (3)</t>
-        </is>
-      </c>
-      <c r="J26" s="313" t="n"/>
-      <c r="K26" s="313" t="inlineStr">
-        <is>
-          <t>0.2617±0.0019 (3)</t>
-        </is>
-      </c>
+      <c r="I26" s="315" t="inlineStr">
+        <is>
+          <t>0.2622±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J26" s="315" t="inlineStr">
+        <is>
+          <t>0.1408±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="K26" s="313" t="n"/>
       <c r="L26" s="313" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="312" t="inlineStr"/>
       <c r="B27" s="312" t="inlineStr">
         <is>
-          <t>raw,d_model 64</t>
+          <t>早期微调配方 large(6k checkpoint)</t>
         </is>
       </c>
       <c r="C27" s="313" t="n"/>
@@ -11872,24 +11868,28 @@
       <c r="F27" s="313" t="n"/>
       <c r="G27" s="313" t="n"/>
       <c r="H27" s="313" t="n"/>
-      <c r="I27" s="313" t="inlineStr">
-        <is>
-          <t>0.3129±0.0121 (3)</t>
-        </is>
-      </c>
-      <c r="J27" s="313" t="n"/>
-      <c r="K27" s="313" t="inlineStr">
-        <is>
-          <t>0.2780±0.0100 (3)</t>
-        </is>
-      </c>
+      <c r="I27" s="315" t="inlineStr">
+        <is>
+          <t>0.2716±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="J27" s="315" t="inlineStr">
+        <is>
+          <t>0.1381±0.0000 (1)</t>
+        </is>
+      </c>
+      <c r="K27" s="313" t="n"/>
       <c r="L27" s="313" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="312" t="inlineStr"/>
+      <c r="A28" s="311" t="inlineStr">
+        <is>
+          <t>容量阶梯</t>
+        </is>
+      </c>
       <c r="B28" s="312" t="inlineStr">
         <is>
-          <t>raw,d_model 256</t>
+          <t>raw,d_model 32</t>
         </is>
       </c>
       <c r="C28" s="313" t="n"/>
@@ -11900,13 +11900,13 @@
       <c r="H28" s="313" t="n"/>
       <c r="I28" s="313" t="inlineStr">
         <is>
-          <t>0.4159±0.0529 (3)</t>
+          <t>0.2613±0.0100 (3)</t>
         </is>
       </c>
       <c r="J28" s="313" t="n"/>
       <c r="K28" s="313" t="inlineStr">
         <is>
-          <t>0.4437±0.0192 (3)</t>
+          <t>0.2617±0.0019 (3)</t>
         </is>
       </c>
       <c r="L28" s="313" t="n"/>
@@ -11915,7 +11915,7 @@
       <c r="A29" s="312" t="inlineStr"/>
       <c r="B29" s="312" t="inlineStr">
         <is>
-          <t>raw,加宽</t>
+          <t>raw,d_model 64</t>
         </is>
       </c>
       <c r="C29" s="313" t="n"/>
@@ -11926,13 +11926,13 @@
       <c r="H29" s="313" t="n"/>
       <c r="I29" s="313" t="inlineStr">
         <is>
-          <t>0.4093±0.0425 (3)</t>
+          <t>0.3129±0.0121 (3)</t>
         </is>
       </c>
       <c r="J29" s="313" t="n"/>
-      <c r="K29" s="315" t="inlineStr">
-        <is>
-          <t>0.4261±0.0085 (2)</t>
+      <c r="K29" s="313" t="inlineStr">
+        <is>
+          <t>0.2780±0.0100 (3)</t>
         </is>
       </c>
       <c r="L29" s="313" t="n"/>
@@ -11941,7 +11941,7 @@
       <c r="A30" s="312" t="inlineStr"/>
       <c r="B30" s="312" t="inlineStr">
         <is>
-          <t>raw,16 频带</t>
+          <t>raw,d_model 256</t>
         </is>
       </c>
       <c r="C30" s="313" t="n"/>
@@ -11952,13 +11952,13 @@
       <c r="H30" s="313" t="n"/>
       <c r="I30" s="313" t="inlineStr">
         <is>
-          <t>0.3781±0.0467 (3)</t>
+          <t>0.4159±0.0529 (3)</t>
         </is>
       </c>
       <c r="J30" s="313" t="n"/>
       <c r="K30" s="313" t="inlineStr">
         <is>
-          <t>0.4288±0.0090 (3)</t>
+          <t>0.4437±0.0192 (3)</t>
         </is>
       </c>
       <c r="L30" s="313" t="n"/>
@@ -11967,7 +11967,7 @@
       <c r="A31" s="312" t="inlineStr"/>
       <c r="B31" s="312" t="inlineStr">
         <is>
-          <t>raw,patch_len 100</t>
+          <t>raw,加宽</t>
         </is>
       </c>
       <c r="C31" s="313" t="n"/>
@@ -11978,13 +11978,13 @@
       <c r="H31" s="313" t="n"/>
       <c r="I31" s="313" t="inlineStr">
         <is>
-          <t>0.3508±0.0251 (3)</t>
+          <t>0.4093±0.0425 (3)</t>
         </is>
       </c>
       <c r="J31" s="313" t="n"/>
-      <c r="K31" s="313" t="inlineStr">
-        <is>
-          <t>0.4066±0.0221 (3)</t>
+      <c r="K31" s="315" t="inlineStr">
+        <is>
+          <t>0.4261±0.0085 (2)</t>
         </is>
       </c>
       <c r="L31" s="313" t="n"/>
@@ -11993,7 +11993,7 @@
       <c r="A32" s="312" t="inlineStr"/>
       <c r="B32" s="312" t="inlineStr">
         <is>
-          <t>raw,dropout 0.5</t>
+          <t>raw,16 频带</t>
         </is>
       </c>
       <c r="C32" s="313" t="n"/>
@@ -12004,13 +12004,13 @@
       <c r="H32" s="313" t="n"/>
       <c r="I32" s="313" t="inlineStr">
         <is>
-          <t>0.3409±0.0196 (3)</t>
+          <t>0.3781±0.0467 (3)</t>
         </is>
       </c>
       <c r="J32" s="313" t="n"/>
       <c r="K32" s="313" t="inlineStr">
         <is>
-          <t>0.4308±0.0139 (3)</t>
+          <t>0.4288±0.0090 (3)</t>
         </is>
       </c>
       <c r="L32" s="313" t="n"/>
@@ -12019,7 +12019,7 @@
       <c r="A33" s="312" t="inlineStr"/>
       <c r="B33" s="312" t="inlineStr">
         <is>
-          <t>raw,attn 头</t>
+          <t>raw,patch_len 100</t>
         </is>
       </c>
       <c r="C33" s="313" t="n"/>
@@ -12030,26 +12030,22 @@
       <c r="H33" s="313" t="n"/>
       <c r="I33" s="313" t="inlineStr">
         <is>
-          <t>0.3524±0.0467 (3)</t>
+          <t>0.3508±0.0251 (3)</t>
         </is>
       </c>
       <c r="J33" s="313" t="n"/>
       <c r="K33" s="313" t="inlineStr">
         <is>
-          <t>0.4545±0.0054 (3)</t>
+          <t>0.4066±0.0221 (3)</t>
         </is>
       </c>
       <c r="L33" s="313" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="311" t="inlineStr">
-        <is>
-          <t>已否决</t>
-        </is>
-      </c>
+      <c r="A34" s="312" t="inlineStr"/>
       <c r="B34" s="312" t="inlineStr">
         <is>
-          <t>spatial_pe: xyz(蒙太奇坐标)</t>
+          <t>raw,dropout 0.5</t>
         </is>
       </c>
       <c r="C34" s="313" t="n"/>
@@ -12057,20 +12053,16 @@
       <c r="E34" s="313" t="n"/>
       <c r="F34" s="313" t="n"/>
       <c r="G34" s="313" t="n"/>
-      <c r="H34" s="313" t="inlineStr">
-        <is>
-          <t>0.6954±0.0167 (3)</t>
-        </is>
-      </c>
+      <c r="H34" s="313" t="n"/>
       <c r="I34" s="313" t="inlineStr">
         <is>
-          <t>0.2478±0.0053 (3)</t>
+          <t>0.3409±0.0196 (3)</t>
         </is>
       </c>
       <c r="J34" s="313" t="n"/>
       <c r="K34" s="313" t="inlineStr">
         <is>
-          <t>0.3338±0.0027 (3)</t>
+          <t>0.4308±0.0139 (3)</t>
         </is>
       </c>
       <c r="L34" s="313" t="n"/>
@@ -12079,7 +12071,7 @@
       <c r="A35" s="312" t="inlineStr"/>
       <c r="B35" s="312" t="inlineStr">
         <is>
-          <t>每窗口归一化</t>
+          <t>raw,attn 头</t>
         </is>
       </c>
       <c r="C35" s="313" t="n"/>
@@ -12090,22 +12082,26 @@
       <c r="H35" s="313" t="n"/>
       <c r="I35" s="313" t="inlineStr">
         <is>
-          <t>0.2532±0.0155 (3)</t>
+          <t>0.3524±0.0467 (3)</t>
         </is>
       </c>
       <c r="J35" s="313" t="n"/>
       <c r="K35" s="313" t="inlineStr">
         <is>
-          <t>0.3050±0.0438 (3)</t>
+          <t>0.4545±0.0054 (3)</t>
         </is>
       </c>
       <c r="L35" s="313" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="312" t="inlineStr"/>
+      <c r="A36" s="311" t="inlineStr">
+        <is>
+          <t>已否决</t>
+        </is>
+      </c>
       <c r="B36" s="312" t="inlineStr">
         <is>
-          <t>每窗口归一化 + raw</t>
+          <t>spatial_pe: xyz(蒙太奇坐标)</t>
         </is>
       </c>
       <c r="C36" s="313" t="n"/>
@@ -12113,16 +12109,20 @@
       <c r="E36" s="313" t="n"/>
       <c r="F36" s="313" t="n"/>
       <c r="G36" s="313" t="n"/>
-      <c r="H36" s="313" t="n"/>
-      <c r="I36" s="315" t="inlineStr">
-        <is>
-          <t>0.2896±0.0146 (2)</t>
+      <c r="H36" s="313" t="inlineStr">
+        <is>
+          <t>0.6954±0.0167 (3)</t>
+        </is>
+      </c>
+      <c r="I36" s="313" t="inlineStr">
+        <is>
+          <t>0.2478±0.0053 (3)</t>
         </is>
       </c>
       <c r="J36" s="313" t="n"/>
-      <c r="K36" s="315" t="inlineStr">
-        <is>
-          <t>0.2992±0.0139 (2)</t>
+      <c r="K36" s="313" t="inlineStr">
+        <is>
+          <t>0.3338±0.0027 (3)</t>
         </is>
       </c>
       <c r="L36" s="313" t="n"/>
@@ -12131,7 +12131,7 @@
       <c r="A37" s="312" t="inlineStr"/>
       <c r="B37" s="312" t="inlineStr">
         <is>
-          <t>每受试者归一化</t>
+          <t>每窗口归一化</t>
         </is>
       </c>
       <c r="C37" s="313" t="n"/>
@@ -12140,20 +12140,24 @@
       <c r="F37" s="313" t="n"/>
       <c r="G37" s="313" t="n"/>
       <c r="H37" s="313" t="n"/>
-      <c r="I37" s="313" t="n"/>
-      <c r="J37" s="315" t="inlineStr">
-        <is>
-          <t>0.1328±0.0007 (2)</t>
-        </is>
-      </c>
-      <c r="K37" s="313" t="n"/>
+      <c r="I37" s="313" t="inlineStr">
+        <is>
+          <t>0.2532±0.0155 (3)</t>
+        </is>
+      </c>
+      <c r="J37" s="313" t="n"/>
+      <c r="K37" s="313" t="inlineStr">
+        <is>
+          <t>0.3050±0.0438 (3)</t>
+        </is>
+      </c>
       <c r="L37" s="313" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="312" t="inlineStr"/>
       <c r="B38" s="312" t="inlineStr">
         <is>
-          <t>每受试者归一化 + raw</t>
+          <t>每窗口归一化 + raw</t>
         </is>
       </c>
       <c r="C38" s="313" t="n"/>
@@ -12162,20 +12166,24 @@
       <c r="F38" s="313" t="n"/>
       <c r="G38" s="313" t="n"/>
       <c r="H38" s="313" t="n"/>
-      <c r="I38" s="313" t="n"/>
-      <c r="J38" s="313" t="inlineStr">
-        <is>
-          <t>0.1579±0.0034 (3)</t>
-        </is>
-      </c>
-      <c r="K38" s="313" t="n"/>
+      <c r="I38" s="315" t="inlineStr">
+        <is>
+          <t>0.2896±0.0146 (2)</t>
+        </is>
+      </c>
+      <c r="J38" s="313" t="n"/>
+      <c r="K38" s="315" t="inlineStr">
+        <is>
+          <t>0.2992±0.0139 (2)</t>
+        </is>
+      </c>
       <c r="L38" s="313" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="312" t="inlineStr"/>
       <c r="B39" s="312" t="inlineStr">
         <is>
-          <t>每受试者归一化 + raw + attn 头</t>
+          <t>每受试者归一化</t>
         </is>
       </c>
       <c r="C39" s="313" t="n"/>
@@ -12185,9 +12193,9 @@
       <c r="G39" s="313" t="n"/>
       <c r="H39" s="313" t="n"/>
       <c r="I39" s="313" t="n"/>
-      <c r="J39" s="313" t="inlineStr">
-        <is>
-          <t>0.1513±0.0012 (3)</t>
+      <c r="J39" s="315" t="inlineStr">
+        <is>
+          <t>0.1328±0.0007 (2)</t>
         </is>
       </c>
       <c r="K39" s="313" t="n"/>
@@ -12197,7 +12205,7 @@
       <c r="A40" s="312" t="inlineStr"/>
       <c r="B40" s="312" t="inlineStr">
         <is>
-          <t>FACED 伪迹清洗</t>
+          <t>每受试者归一化 + raw</t>
         </is>
       </c>
       <c r="C40" s="313" t="n"/>
@@ -12209,7 +12217,7 @@
       <c r="I40" s="313" t="n"/>
       <c r="J40" s="313" t="inlineStr">
         <is>
-          <t>0.1346±0.0157 (3)</t>
+          <t>0.1579±0.0034 (3)</t>
         </is>
       </c>
       <c r="K40" s="313" t="n"/>
@@ -12219,7 +12227,7 @@
       <c r="A41" s="312" t="inlineStr"/>
       <c r="B41" s="312" t="inlineStr">
         <is>
-          <t>lr 1e-3</t>
+          <t>每受试者归一化 + raw + attn 头</t>
         </is>
       </c>
       <c r="C41" s="313" t="n"/>
@@ -12228,24 +12236,20 @@
       <c r="F41" s="313" t="n"/>
       <c r="G41" s="313" t="n"/>
       <c r="H41" s="313" t="n"/>
-      <c r="I41" s="313" t="inlineStr">
-        <is>
-          <t>0.2498±0.0077 (3)</t>
-        </is>
-      </c>
-      <c r="J41" s="313" t="n"/>
-      <c r="K41" s="313" t="inlineStr">
-        <is>
-          <t>0.3094±0.0345 (3)</t>
-        </is>
-      </c>
+      <c r="I41" s="313" t="n"/>
+      <c r="J41" s="313" t="inlineStr">
+        <is>
+          <t>0.1513±0.0012 (3)</t>
+        </is>
+      </c>
+      <c r="K41" s="313" t="n"/>
       <c r="L41" s="313" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="312" t="inlineStr"/>
       <c r="B42" s="312" t="inlineStr">
         <is>
-          <t>lr 3e-4</t>
+          <t>FACED 伪迹清洗</t>
         </is>
       </c>
       <c r="C42" s="313" t="n"/>
@@ -12254,155 +12258,203 @@
       <c r="F42" s="313" t="n"/>
       <c r="G42" s="313" t="n"/>
       <c r="H42" s="313" t="n"/>
-      <c r="I42" s="313" t="inlineStr">
-        <is>
-          <t>0.2623±0.0042 (3)</t>
-        </is>
-      </c>
-      <c r="J42" s="313" t="n"/>
-      <c r="K42" s="313" t="inlineStr">
-        <is>
-          <t>0.3495±0.0039 (3)</t>
-        </is>
-      </c>
+      <c r="I42" s="313" t="n"/>
+      <c r="J42" s="313" t="inlineStr">
+        <is>
+          <t>0.1346±0.0157 (3)</t>
+        </is>
+      </c>
+      <c r="K42" s="313" t="n"/>
       <c r="L42" s="313" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="311" t="inlineStr">
-        <is>
-          <t>早期 pilot</t>
-        </is>
-      </c>
+      <c r="A43" s="312" t="inlineStr"/>
       <c r="B43" s="312" t="inlineStr">
         <is>
-          <t>冻结前端 pilot</t>
+          <t>lr 1e-3</t>
         </is>
       </c>
       <c r="C43" s="313" t="n"/>
-      <c r="D43" s="313" t="inlineStr">
-        <is>
-          <t>0.6272±0.0099 (3)</t>
-        </is>
-      </c>
+      <c r="D43" s="313" t="n"/>
       <c r="E43" s="313" t="n"/>
       <c r="F43" s="313" t="n"/>
       <c r="G43" s="313" t="n"/>
       <c r="H43" s="313" t="n"/>
-      <c r="I43" s="313" t="n"/>
+      <c r="I43" s="313" t="inlineStr">
+        <is>
+          <t>0.2498±0.0077 (3)</t>
+        </is>
+      </c>
       <c r="J43" s="313" t="n"/>
-      <c r="K43" s="313" t="n"/>
+      <c r="K43" s="313" t="inlineStr">
+        <is>
+          <t>0.3094±0.0345 (3)</t>
+        </is>
+      </c>
       <c r="L43" s="313" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="312" t="inlineStr"/>
       <c r="B44" s="312" t="inlineStr">
         <is>
-          <t>未滤波 pilot</t>
+          <t>lr 3e-4</t>
         </is>
       </c>
       <c r="C44" s="313" t="n"/>
-      <c r="D44" s="313" t="inlineStr">
-        <is>
-          <t>0.6209±0.0503 (3)</t>
-        </is>
-      </c>
+      <c r="D44" s="313" t="n"/>
       <c r="E44" s="313" t="n"/>
       <c r="F44" s="313" t="n"/>
       <c r="G44" s="313" t="n"/>
       <c r="H44" s="313" t="n"/>
-      <c r="I44" s="313" t="n"/>
+      <c r="I44" s="313" t="inlineStr">
+        <is>
+          <t>0.2623±0.0042 (3)</t>
+        </is>
+      </c>
       <c r="J44" s="313" t="n"/>
-      <c r="K44" s="313" t="n"/>
+      <c r="K44" s="313" t="inlineStr">
+        <is>
+          <t>0.3495±0.0039 (3)</t>
+        </is>
+      </c>
       <c r="L44" s="313" t="n"/>
     </row>
+    <row r="45">
+      <c r="A45" s="311" t="inlineStr">
+        <is>
+          <t>早期 pilot</t>
+        </is>
+      </c>
+      <c r="B45" s="312" t="inlineStr">
+        <is>
+          <t>冻结前端 pilot</t>
+        </is>
+      </c>
+      <c r="C45" s="313" t="n"/>
+      <c r="D45" s="313" t="inlineStr">
+        <is>
+          <t>0.6272±0.0099 (3)</t>
+        </is>
+      </c>
+      <c r="E45" s="313" t="n"/>
+      <c r="F45" s="313" t="n"/>
+      <c r="G45" s="313" t="n"/>
+      <c r="H45" s="313" t="n"/>
+      <c r="I45" s="313" t="n"/>
+      <c r="J45" s="313" t="n"/>
+      <c r="K45" s="313" t="n"/>
+      <c r="L45" s="313" t="n"/>
+    </row>
     <row r="46">
-      <c r="A46" s="316" t="inlineStr">
+      <c r="A46" s="312" t="inlineStr"/>
+      <c r="B46" s="312" t="inlineStr">
+        <is>
+          <t>未滤波 pilot</t>
+        </is>
+      </c>
+      <c r="C46" s="313" t="n"/>
+      <c r="D46" s="313" t="inlineStr">
+        <is>
+          <t>0.6209±0.0503 (3)</t>
+        </is>
+      </c>
+      <c r="E46" s="313" t="n"/>
+      <c r="F46" s="313" t="n"/>
+      <c r="G46" s="313" t="n"/>
+      <c r="H46" s="313" t="n"/>
+      <c r="I46" s="313" t="n"/>
+      <c r="J46" s="313" t="n"/>
+      <c r="K46" s="313" t="n"/>
+      <c r="L46" s="313" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="316" t="inlineStr">
         <is>
           <t>样本量消融</t>
         </is>
       </c>
-      <c r="B46" s="317" t="inlineStr">
+      <c r="B48" s="317" t="inlineStr">
         <is>
           <t>TUEV 训练集降采样(kappa) —— 检验等级三是否只是样本量问题</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="309" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="309" t="inlineStr">
         <is>
           <t>模型</t>
         </is>
       </c>
-      <c r="C47" s="310" t="inlineStr">
+      <c r="C49" s="310" t="inlineStr">
         <is>
           <t>n=2160</t>
         </is>
       </c>
-      <c r="D47" s="310" t="inlineStr">
+      <c r="D49" s="310" t="inlineStr">
         <is>
           <t>n=6720</t>
         </is>
       </c>
-      <c r="E47" s="310" t="inlineStr">
+      <c r="E49" s="310" t="inlineStr">
         <is>
           <t>n=20000</t>
         </is>
       </c>
-      <c r="F47" s="310" t="inlineStr">
+      <c r="F49" s="310" t="inlineStr">
         <is>
           <t>全量 68445</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="312" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="312" t="inlineStr">
         <is>
           <t>PACLock v2</t>
         </is>
       </c>
-      <c r="C48" s="315" t="inlineStr">
+      <c r="C50" s="315" t="inlineStr">
         <is>
           <t>0.6523±0.0000 (1)</t>
         </is>
       </c>
-      <c r="D48" s="315" t="inlineStr">
+      <c r="D50" s="315" t="inlineStr">
         <is>
           <t>0.7098±0.0000 (1)</t>
         </is>
       </c>
-      <c r="E48" s="315" t="inlineStr">
+      <c r="E50" s="315" t="inlineStr">
         <is>
           <t>0.6767±0.0000 (1)</t>
         </is>
       </c>
-      <c r="F48" s="313" t="inlineStr">
+      <c r="F50" s="313" t="inlineStr">
         <is>
           <t>0.7076±0.0311 (3)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="312" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="312" t="inlineStr">
         <is>
           <t>SPaRCNet</t>
         </is>
       </c>
-      <c r="C49" s="315" t="inlineStr">
+      <c r="C51" s="315" t="inlineStr">
         <is>
           <t>0.4917±0.0000 (1)</t>
         </is>
       </c>
-      <c r="D49" s="315" t="inlineStr">
+      <c r="D51" s="315" t="inlineStr">
         <is>
           <t>0.5532±0.0000 (1)</t>
         </is>
       </c>
-      <c r="E49" s="315" t="inlineStr">
+      <c r="E51" s="315" t="inlineStr">
         <is>
           <t>0.3642±0.0000 (1)</t>
         </is>
       </c>
-      <c r="F49" s="313" t="inlineStr">
+      <c r="F51" s="313" t="inlineStr">
         <is>
           <t>0.4885±0.0279 (3)</t>
         </is>

</xml_diff>

<commit_message>
Workbook: pretraining-diagnostics sheet (probes, label fraction, Siena per-subject, tune winners)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/PACLock_baseline_matrix_filled.xlsx
+++ b/results/PACLock_baseline_matrix_filled.xlsx
@@ -27,6 +27,7 @@
     <sheet name="EEGMat" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="_填写记录" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="_消融" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="_预训练诊断" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1343,7 +1344,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -1915,7 +1915,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -2451,7 +2450,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -3023,7 +3021,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -3541,7 +3538,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -4041,7 +4037,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -4613,7 +4608,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -5203,7 +5197,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -5775,7 +5768,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -27670,7 +27662,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -27712,7 +27703,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
@@ -29301,6 +29291,632 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>预训练诊断(2026-09-02 定稿;结论见 docs/FINDINGS.md 5.6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>A. 冻结探针,lr=1e-3(与参考线匹配)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>checkpoint</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>TUSZ pr_auc</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>TUEV kappa</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>随机初始化</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.4076</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.3859</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>v1 欠训 1.6ep</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.4842</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.6351</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>v2 欠训 1.6ep</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.5417</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5184</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>v2 收敛 15.4ep (ptF)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.4445275840076715</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.6509876244558666</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>v3(FAME) 20k</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3328237539130039</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.5391831434368992</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>v3(FAME) 40k</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.4112430646733859</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.5496358730083497</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>v3(FAME) 60k</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.3836310517716551</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.4708963361620297</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>v3(FAME) 80k</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.4718484877398866</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.5319707988149562</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>v3(FAME) 100k</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.5047550940108541</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.5639229466028473</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>A2. 同上,lr=1e-4(内部对照组,不与参考线比)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>v2 收敛 (ptF)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.5813</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>v3(FAME) 20k</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.397958610027846</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.4715749021437604</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>v3(FAME) 40k</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.4911939914046341</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.3708686448909037</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>v3(FAME) 60k</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.2777385287081304</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.4875331791018003</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>v3(FAME) 80k</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.4883372136553454</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.5155547316871869</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>v3(FAME) 100k</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.4924195988451215</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.5144236053003975</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>B. 标注量消融(scratch vs ptF,单 seed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>语料</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>训练量</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>scratch</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>ptF</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>tusz</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>05%</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.6409847213931373</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.5777148438818177</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-0.06326987751131963</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>tusz</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.5306988364843777</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.5821092683396684</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.05141043185529071</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>tusz</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.5688782571777783</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.5916386242776533</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.02276036709987506</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>tusz</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.6328</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.4968</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-0.136</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>tuev</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>05%</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0.5411598657522759</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.5205810950586779</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-0.02057877069359804</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>tuev</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0.6936138339658515</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.5747054109455207</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-0.1189084230203308</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tuev</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0.7304827265373887</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.598865761794396</v>
+      </c>
+      <c r="E31" t="n">
+        <v>-0.1316169647429927</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tuev</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0.7094</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.5662</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-0.1432</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>C. Siena 逐被试 AP(配方匹配对:32x4/60ep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>被试</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>scratch</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>ptF</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PN14</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.0159</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.1276</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PN16</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.0304</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.5852000000000001</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PN17</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.3515</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.7725</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>全局</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.0654</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.4682</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>D. 调参探针赢家(val 选优;赢家将于定稿波升为格子配方)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>语料</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>arm</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>旧格子值</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>caueeg</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>paclock_tune_t3</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>0.5577902721924565</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.5254</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>mumtaz</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>paclock_tune_t1</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>0.9804125177809389</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.9775</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>tuar</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>paclock_tune_t1</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>0.6575608887426647</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.6289</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>adfd</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>paclock_ptF_lr3rd</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>0.4824716290965309</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.3786</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -29961,7 +30577,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -30616,7 +31231,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -31224,7 +31838,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -31879,7 +32492,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -32516,7 +33128,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -32558,7 +33169,6 @@
         </is>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
@@ -33195,7 +33805,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -33785,7 +34394,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
@@ -33798,7 +34406,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>

</xml_diff>